<commit_message>
1. update ethercat xml file 2. modify files in bgm_app folder 3. optimize code
</commit_message>
<xml_diff>
--- a/ArmCoreV1_QSPI/SSCProject/lan9252_app.xlsx
+++ b/ArmCoreV1_QSPI/SSCProject/lan9252_app.xlsx
@@ -1,20 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\WORK\arm_core_develop\bgm_arm_io_develop\FW-ArmCore\ArmCoreV1_QSPI\SSCProject\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView windowHeight="17655"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="17660"/>
   </bookViews>
   <sheets>
     <sheet name="Profile" sheetId="11" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Profile!$B$10:$P$61</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Profile!$B$1:$P$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Profile!$B$10:$P$76</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Profile!$B$1:$P$77</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -32,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="96">
   <si>
     <t>Device Profile:</t>
   </si>
@@ -308,107 +313,508 @@
     <t>USINT</t>
   </si>
   <si>
-    <t>InU8_Test1</t>
-  </si>
-  <si>
-    <t>BOOL</t>
-  </si>
-  <si>
-    <t>InB1_Test2</t>
-  </si>
-  <si>
-    <t>BIT7</t>
-  </si>
-  <si>
-    <t>InB7_Test3</t>
-  </si>
-  <si>
     <t>UINT</t>
   </si>
   <si>
-    <t>InU16_Test4</t>
+    <t>//0x7nnx</t>
+  </si>
+  <si>
+    <t>Output Data of the Module (0x7000 - 0x7FFF)</t>
+  </si>
+  <si>
+    <t>0x7010</t>
+  </si>
+  <si>
+    <t>OutputData</t>
+  </si>
+  <si>
+    <t>//0x8nnx</t>
+  </si>
+  <si>
+    <t>Configuration Data of the Module (0x8000 - 0x8FFF)</t>
+  </si>
+  <si>
+    <t>//0x9nnx</t>
+  </si>
+  <si>
+    <t>Information Data of the Module (0x9000 - 0x9FFF)</t>
+  </si>
+  <si>
+    <t>//0xAnnx</t>
+  </si>
+  <si>
+    <t>Diagnosis Data of the Module (0xA000 - 0xAFFF)</t>
+  </si>
+  <si>
+    <r>
+      <t>InU16_Ra</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>diationIndex</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SINT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_FsmState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>INT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nU16_NotReadyEvent</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DINT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>In</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>U32_WaringInterlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nU32_MinorInterlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_SeriousInterlock</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>R</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EAL</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_PrimaryDoseTotalActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_SecondaryDoseTotalActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_PrimaryDoseRateActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_SecondaryDoseRateActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RM IO FSM State</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RM IO Interlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_DoseAInterlock</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>InU32_Dose</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Interlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DOSEA</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DOSEB</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DOSEB</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>REAL</t>
-  </si>
-  <si>
-    <t>InF_Test5</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_DoseAFsmState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_DoseBFsmState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DINT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>R</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EAL</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_AfcPositionCurrent</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>OutU8_RequireState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utU8_BeamId</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>InU8_BeamI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>d</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utU16_RadiationIndex</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>R</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EAL</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utF_GantryPosition</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
     <t>UDINT</t>
-  </si>
-  <si>
-    <t>InU32_Test6</t>
-  </si>
-  <si>
-    <t>LREAL</t>
-  </si>
-  <si>
-    <t>InD_Test7</t>
-  </si>
-  <si>
-    <t>//0x7nnx</t>
-  </si>
-  <si>
-    <t>Output Data of the Module (0x7000 - 0x7FFF)</t>
-  </si>
-  <si>
-    <t>0x7010</t>
-  </si>
-  <si>
-    <t>OutputData</t>
-  </si>
-  <si>
-    <t>OutU8_Test1</t>
-  </si>
-  <si>
-    <t>OutB1_Test2</t>
-  </si>
-  <si>
-    <t>OutB7_Test3</t>
-  </si>
-  <si>
-    <t>OutU16_Test4</t>
-  </si>
-  <si>
-    <t>OutF_Test5</t>
-  </si>
-  <si>
-    <t>OutU32_Test6</t>
-  </si>
-  <si>
-    <t>OutD_Test7</t>
-  </si>
-  <si>
-    <t>//0x8nnx</t>
-  </si>
-  <si>
-    <t>Configuration Data of the Module (0x8000 - 0x8FFF)</t>
-  </si>
-  <si>
-    <t>//0x9nnx</t>
-  </si>
-  <si>
-    <t>Information Data of the Module (0x9000 - 0x9FFF)</t>
-  </si>
-  <si>
-    <t>//0xAnnx</t>
-  </si>
-  <si>
-    <t>Diagnosis Data of the Module (0xA000 - 0xAFFF)</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>UDINT</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>OutU32_InterlockOverride</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>OutU32_UnreadyOveride</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>REAL</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_BeamOnTime</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">ARM IO First Trigger Out start count </t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>UDINT</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_AfcState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="23">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -439,151 +845,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
+      <sz val="9"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -592,210 +868,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.349986266670736"/>
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.149998474074526"/>
+        <fgColor theme="0" tint="-0.14996795556505021"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.15"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -803,253 +893,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
@@ -1063,9 +911,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -1102,62 +947,24 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1444,33 +1251,33 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:T912"/>
-  <sheetFormatPr defaultColWidth="10.7079646017699" defaultRowHeight="13.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:T927"/>
+  <sheetFormatPr defaultColWidth="10.7265625" defaultRowHeight="14" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="3.85840707964602" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.283185840708" style="2" customWidth="1"/>
-    <col min="3" max="4" width="14.7079646017699" style="2" customWidth="1"/>
-    <col min="5" max="5" width="22.1858407079646" style="2" customWidth="1"/>
-    <col min="6" max="6" width="40.7079646017699" style="2" customWidth="1"/>
-    <col min="7" max="7" width="11.7079646017699" style="2" customWidth="1"/>
-    <col min="8" max="9" width="7.70796460176991" style="2" customWidth="1"/>
-    <col min="10" max="10" width="10.283185840708" style="2" customWidth="1"/>
-    <col min="11" max="11" width="7.70796460176991" style="2" customWidth="1"/>
-    <col min="12" max="12" width="11.7079646017699" style="2" customWidth="1"/>
-    <col min="13" max="13" width="7.70796460176991" style="2" customWidth="1"/>
-    <col min="14" max="14" width="11.7079646017699" style="2" customWidth="1"/>
-    <col min="15" max="15" width="11.858407079646" style="2" customWidth="1"/>
-    <col min="16" max="16" width="35.7079646017699" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="10.7079646017699" style="2"/>
+    <col min="1" max="1" width="3.81640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.26953125" style="2" customWidth="1"/>
+    <col min="3" max="4" width="14.7265625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="22.1796875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="40.7265625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="11.7265625" style="2" customWidth="1"/>
+    <col min="8" max="9" width="7.7265625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="10.26953125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="7.7265625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="11.7265625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="7.7265625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="11.7265625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="11.81640625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="43.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="10.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" spans="1:20">
+    <row r="1" spans="1:20" ht="18.75" customHeight="1">
       <c r="A1" s="3"/>
       <c r="B1" s="4" t="s">
         <v>0</v>
@@ -1482,93 +1289,93 @@
         <v>1</v>
       </c>
       <c r="E1" s="4"/>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="21"/>
-      <c r="T1" s="21"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" s="3"/>
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="20"/>
+      <c r="R2" s="20"/>
+      <c r="S2" s="20"/>
+      <c r="T2" s="20"/>
     </row>
     <row r="3" spans="1:20">
       <c r="A3" s="3"/>
-      <c r="B3" s="8"/>
+      <c r="B3" s="7"/>
       <c r="C3" s="5"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="21"/>
-      <c r="R3" s="21"/>
-      <c r="S3" s="21"/>
-      <c r="T3" s="21"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="20"/>
+      <c r="R3" s="20"/>
+      <c r="S3" s="20"/>
+      <c r="T3" s="20"/>
     </row>
     <row r="4" spans="1:20">
       <c r="A4" s="3"/>
-      <c r="B4" s="8"/>
+      <c r="B4" s="7"/>
       <c r="C4" s="5"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="21"/>
-      <c r="R4" s="21"/>
-      <c r="S4" s="21"/>
-      <c r="T4" s="21"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="3"/>
@@ -1576,21 +1383,21 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="21"/>
-      <c r="T5" s="21"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
     </row>
     <row r="6" spans="1:20">
       <c r="A6" s="3"/>
@@ -1598,21 +1405,21 @@
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="21"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
+      <c r="S6" s="20"/>
+      <c r="T6" s="20"/>
     </row>
     <row r="7" spans="1:20">
       <c r="A7" s="3"/>
@@ -1620,25 +1427,25 @@
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="21"/>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
+    </row>
+    <row r="8" spans="1:20">
       <c r="A8" s="3"/>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="4"/>
@@ -1656,7 +1463,7 @@
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:20">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1674,539 +1481,539 @@
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:20">
       <c r="A10" s="3"/>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="K10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="L10" s="11" t="s">
+      <c r="L10" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="M10" s="11" t="s">
+      <c r="M10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="N10" s="20" t="s">
+      <c r="N10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="O10" s="20" t="s">
+      <c r="O10" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="P10" s="11" t="s">
+      <c r="P10" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" spans="1:16">
-      <c r="A11" s="12"/>
-      <c r="B11" s="13" t="s">
+    <row r="11" spans="1:20" s="1" customFormat="1">
+      <c r="A11" s="11"/>
+      <c r="B11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+    </row>
+    <row r="12" spans="1:20">
       <c r="A12" s="3"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="14"/>
-      <c r="O12" s="14"/>
-      <c r="P12" s="16"/>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="15"/>
+    </row>
+    <row r="13" spans="1:20">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
-      <c r="P13" s="12"/>
-    </row>
-    <row r="14" s="1" customFormat="1" spans="1:16">
-      <c r="A14" s="12"/>
-      <c r="B14" s="18" t="s">
+      <c r="P13" s="11"/>
+    </row>
+    <row r="14" spans="1:20" s="1" customFormat="1">
+      <c r="A14" s="11"/>
+      <c r="B14" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="18"/>
-      <c r="P14" s="18"/>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+    </row>
+    <row r="15" spans="1:20">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
-      <c r="P15" s="12"/>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="P15" s="11"/>
+    </row>
+    <row r="16" spans="1:20">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
-      <c r="P16" s="12"/>
-    </row>
-    <row r="17" s="1" customFormat="1" hidden="1" outlineLevel="1" spans="1:16">
-      <c r="A17" s="12"/>
-      <c r="B17" s="18" t="s">
+      <c r="P16" s="11"/>
+    </row>
+    <row r="17" spans="1:16" s="1" customFormat="1" hidden="1" outlineLevel="1">
+      <c r="A17" s="11"/>
+      <c r="B17" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
-      <c r="N17" s="18"/>
-      <c r="O17" s="18"/>
-      <c r="P17" s="18"/>
-    </row>
-    <row r="18" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="17"/>
+    </row>
+    <row r="18" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
-      <c r="P18" s="12"/>
-    </row>
-    <row r="19" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="P18" s="11"/>
+    </row>
+    <row r="19" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
-      <c r="P19" s="12"/>
-    </row>
-    <row r="20" s="1" customFormat="1" hidden="1" outlineLevel="1" spans="1:16">
-      <c r="A20" s="12"/>
-      <c r="B20" s="18" t="s">
+      <c r="P19" s="11"/>
+    </row>
+    <row r="20" spans="1:16" s="1" customFormat="1" hidden="1" outlineLevel="1">
+      <c r="A20" s="11"/>
+      <c r="B20" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="18"/>
-      <c r="N20" s="18"/>
-      <c r="O20" s="18"/>
-      <c r="P20" s="18"/>
-    </row>
-    <row r="21" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+    </row>
+    <row r="21" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="12"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
-      <c r="P21" s="12"/>
-    </row>
-    <row r="22" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="P21" s="11"/>
+    </row>
+    <row r="22" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
       <c r="O22" s="3"/>
-      <c r="P22" s="12"/>
-    </row>
-    <row r="23" s="1" customFormat="1" hidden="1" outlineLevel="1" spans="1:16">
-      <c r="A23" s="12"/>
-      <c r="B23" s="18" t="s">
+      <c r="P22" s="11"/>
+    </row>
+    <row r="23" spans="1:16" s="1" customFormat="1" hidden="1" outlineLevel="1">
+      <c r="A23" s="11"/>
+      <c r="B23" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="18"/>
-      <c r="N23" s="18"/>
-      <c r="O23" s="18"/>
-      <c r="P23" s="18"/>
-    </row>
-    <row r="24" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+    </row>
+    <row r="24" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="12"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
-      <c r="P24" s="12"/>
-    </row>
-    <row r="25" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="P24" s="11"/>
+    </row>
+    <row r="25" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
-      <c r="P25" s="12"/>
-    </row>
-    <row r="26" s="1" customFormat="1" hidden="1" outlineLevel="1" spans="1:16">
-      <c r="A26" s="12"/>
-      <c r="B26" s="18" t="s">
+      <c r="P25" s="11"/>
+    </row>
+    <row r="26" spans="1:16" s="1" customFormat="1" hidden="1" outlineLevel="1">
+      <c r="A26" s="11"/>
+      <c r="B26" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="18"/>
-      <c r="N26" s="18"/>
-      <c r="O26" s="18"/>
-      <c r="P26" s="18"/>
-    </row>
-    <row r="27" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="17"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="17"/>
+      <c r="P26" s="17"/>
+    </row>
+    <row r="27" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
-      <c r="P27" s="12"/>
-    </row>
-    <row r="28" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="P27" s="11"/>
+    </row>
+    <row r="28" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="12"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
-      <c r="P28" s="12"/>
-    </row>
-    <row r="29" s="1" customFormat="1" hidden="1" outlineLevel="1" spans="1:16">
-      <c r="A29" s="12"/>
-      <c r="B29" s="18" t="s">
+      <c r="P28" s="11"/>
+    </row>
+    <row r="29" spans="1:16" s="1" customFormat="1" hidden="1" outlineLevel="1">
+      <c r="A29" s="11"/>
+      <c r="B29" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="18"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="18"/>
-      <c r="N29" s="18"/>
-      <c r="O29" s="18"/>
-      <c r="P29" s="18"/>
-    </row>
-    <row r="30" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="17"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="17"/>
+      <c r="O29" s="17"/>
+      <c r="P29" s="17"/>
+    </row>
+    <row r="30" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
-      <c r="I30" s="12"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
-      <c r="P30" s="12"/>
-    </row>
-    <row r="31" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="P30" s="11"/>
+    </row>
+    <row r="31" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="12"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
-      <c r="P31" s="12"/>
-    </row>
-    <row r="32" s="1" customFormat="1" hidden="1" outlineLevel="1" spans="1:16">
-      <c r="A32" s="12"/>
-      <c r="B32" s="18" t="s">
+      <c r="P31" s="11"/>
+    </row>
+    <row r="32" spans="1:16" s="1" customFormat="1" hidden="1" outlineLevel="1">
+      <c r="A32" s="11"/>
+      <c r="B32" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="O32" s="18"/>
-      <c r="P32" s="18"/>
-    </row>
-    <row r="33" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="17"/>
+      <c r="L32" s="17"/>
+      <c r="M32" s="17"/>
+      <c r="N32" s="17"/>
+      <c r="O32" s="17"/>
+      <c r="P32" s="17"/>
+    </row>
+    <row r="33" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
-      <c r="I33" s="12"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
-      <c r="P33" s="12"/>
-    </row>
-    <row r="34" hidden="1" outlineLevel="1" spans="1:16">
+      <c r="P33" s="11"/>
+    </row>
+    <row r="34" spans="1:16" hidden="1" outlineLevel="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
-      <c r="I34" s="12"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
-      <c r="P34" s="12"/>
-    </row>
-    <row r="35" s="1" customFormat="1" collapsed="1" spans="1:16">
-      <c r="A35" s="12"/>
-      <c r="B35" s="18" t="s">
+      <c r="P34" s="11"/>
+    </row>
+    <row r="35" spans="1:16" s="1" customFormat="1" collapsed="1">
+      <c r="A35" s="11"/>
+      <c r="B35" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="18"/>
-      <c r="K35" s="18"/>
-      <c r="L35" s="18"/>
-      <c r="M35" s="18"/>
-      <c r="N35" s="18"/>
-      <c r="O35" s="18"/>
-      <c r="P35" s="18"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+      <c r="L35" s="17"/>
+      <c r="M35" s="17"/>
+      <c r="N35" s="17"/>
+      <c r="O35" s="17"/>
+      <c r="P35" s="17"/>
     </row>
     <row r="36" spans="1:16">
       <c r="A36" s="3"/>
@@ -2216,854 +2023,1151 @@
       <c r="C36" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="17"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12" t="s">
+      <c r="D36" s="16"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="12"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
       <c r="N36" s="3"/>
       <c r="O36" s="3"/>
-      <c r="P36" s="12"/>
-    </row>
-    <row r="37" customFormat="1" spans="1:16">
+      <c r="P36" s="11"/>
+    </row>
+    <row r="37" spans="1:16" customFormat="1">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
-      <c r="D37" s="17">
+      <c r="D37" s="16">
         <v>1</v>
       </c>
-      <c r="E37" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F37" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
+      <c r="E37" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F37" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
       <c r="N37" s="3"/>
       <c r="O37" s="3"/>
-      <c r="P37" s="12"/>
-    </row>
-    <row r="38" customFormat="1" spans="1:16">
+      <c r="P37" s="21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" customFormat="1">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
-      <c r="D38" s="17">
+      <c r="D38" s="16">
         <v>2</v>
       </c>
-      <c r="E38" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="12"/>
+      <c r="E38" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F38" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
-      <c r="P38" s="12"/>
-    </row>
-    <row r="39" customFormat="1" spans="1:16">
+      <c r="P38" s="11"/>
+    </row>
+    <row r="39" spans="1:16" customFormat="1">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
-      <c r="D39" s="17">
+      <c r="D39" s="16">
         <v>3</v>
       </c>
-      <c r="E39" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="F39" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="12"/>
+      <c r="E39" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F39" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
-      <c r="P39" s="12"/>
-    </row>
-    <row r="40" customFormat="1" spans="1:16">
-      <c r="A40" s="3">
-        <v>4</v>
-      </c>
+      <c r="P39" s="11"/>
+    </row>
+    <row r="40" spans="1:16" customFormat="1">
+      <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
-      <c r="D40" s="17">
+      <c r="D40" s="16">
         <v>4</v>
       </c>
-      <c r="E40" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F40" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="12"/>
+      <c r="E40" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="F40" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
-      <c r="P40" s="12"/>
-    </row>
-    <row r="41" customFormat="1" spans="1:16">
+      <c r="P40" s="11"/>
+    </row>
+    <row r="41" spans="1:16" customFormat="1">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
-      <c r="D41" s="17">
+      <c r="D41" s="16">
         <v>5</v>
       </c>
-      <c r="E41" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="G41" s="12"/>
-      <c r="H41" s="12"/>
-      <c r="I41" s="12"/>
+      <c r="E41" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F41" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+      <c r="I41" s="11"/>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
       <c r="N41" s="3"/>
       <c r="O41" s="3"/>
-      <c r="P41" s="12"/>
-    </row>
-    <row r="42" customFormat="1" spans="1:16">
+      <c r="P41" s="11"/>
+    </row>
+    <row r="42" spans="1:16" customFormat="1">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
-      <c r="D42" s="17">
+      <c r="D42" s="16">
         <v>6</v>
       </c>
-      <c r="E42" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="G42" s="12"/>
-      <c r="H42" s="12"/>
-      <c r="I42" s="12"/>
+      <c r="E42" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F42" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G42" s="11"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="11"/>
       <c r="J42" s="3"/>
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
       <c r="N42" s="3"/>
       <c r="O42" s="3"/>
-      <c r="P42" s="12"/>
-    </row>
-    <row r="43" customFormat="1" spans="1:16">
+      <c r="P42" s="11"/>
+    </row>
+    <row r="43" spans="1:16" customFormat="1">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
-      <c r="D43" s="17">
+      <c r="D43" s="16">
         <v>7</v>
       </c>
-      <c r="E43" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F43" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="G43" s="12"/>
-      <c r="H43" s="12"/>
-      <c r="I43" s="12"/>
+      <c r="E43" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F43" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="G43" s="11"/>
+      <c r="H43" s="11"/>
+      <c r="I43" s="11"/>
       <c r="J43" s="3"/>
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
       <c r="N43" s="3"/>
       <c r="O43" s="3"/>
-      <c r="P43" s="12"/>
-    </row>
-    <row r="44" s="1" customFormat="1" spans="1:16">
-      <c r="A44" s="12"/>
-      <c r="B44" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
-      <c r="F44" s="18"/>
-      <c r="G44" s="18"/>
-      <c r="H44" s="18"/>
-      <c r="I44" s="18"/>
-      <c r="J44" s="18"/>
-      <c r="K44" s="18"/>
-      <c r="L44" s="18"/>
-      <c r="M44" s="18"/>
-      <c r="N44" s="18"/>
-      <c r="O44" s="18"/>
-      <c r="P44" s="18"/>
-    </row>
-    <row r="45" spans="1:16">
+      <c r="P43" s="21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" customFormat="1">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="16">
+        <v>8</v>
+      </c>
+      <c r="E44" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="F44" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="G44" s="11"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="11"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+      <c r="P44" s="21" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" customFormat="1">
       <c r="A45" s="3"/>
-      <c r="B45" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D45" s="17"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
-      <c r="I45" s="12"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="16">
+        <v>9</v>
+      </c>
+      <c r="E45" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="F45" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="G45" s="11"/>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11"/>
       <c r="J45" s="3"/>
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
       <c r="N45" s="3"/>
       <c r="O45" s="3"/>
-      <c r="P45" s="12"/>
-    </row>
-    <row r="46" customFormat="1" spans="1:16">
+      <c r="P45" s="21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" customFormat="1">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
-      <c r="D46" s="17">
-        <v>1</v>
-      </c>
-      <c r="E46" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F46" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="G46" s="12"/>
-      <c r="H46" s="12"/>
-      <c r="I46" s="12"/>
+      <c r="D46" s="16">
+        <v>10</v>
+      </c>
+      <c r="E46" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="F46" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11"/>
       <c r="J46" s="3"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
       <c r="N46" s="3"/>
       <c r="O46" s="3"/>
-      <c r="P46" s="12"/>
-    </row>
-    <row r="47" customFormat="1" spans="1:16">
+      <c r="P46" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" customFormat="1">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
-      <c r="D47" s="17">
-        <v>2</v>
-      </c>
-      <c r="E47" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="12"/>
+      <c r="D47" s="16">
+        <v>11</v>
+      </c>
+      <c r="E47" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="F47" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="G47" s="11"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
       <c r="J47" s="3"/>
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3"/>
       <c r="N47" s="3"/>
       <c r="O47" s="3"/>
-      <c r="P47" s="12"/>
-    </row>
-    <row r="48" customFormat="1" spans="1:16">
+      <c r="P47" s="21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" customFormat="1">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
-      <c r="D48" s="17">
-        <v>3</v>
-      </c>
-      <c r="E48" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="F48" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="G48" s="12"/>
-      <c r="H48" s="12"/>
-      <c r="I48" s="12"/>
+      <c r="D48" s="16">
+        <v>12</v>
+      </c>
+      <c r="E48" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="F48" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="G48" s="11"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
       <c r="J48" s="3"/>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
       <c r="N48" s="3"/>
       <c r="O48" s="3"/>
-      <c r="P48" s="12"/>
-    </row>
-    <row r="49" customFormat="1" spans="1:16">
+      <c r="P48" s="21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" customFormat="1">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
-      <c r="D49" s="17">
-        <v>4</v>
-      </c>
-      <c r="E49" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="F49" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="G49" s="12"/>
-      <c r="H49" s="12"/>
-      <c r="I49" s="12"/>
+      <c r="D49" s="16">
+        <v>13</v>
+      </c>
+      <c r="E49" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F49" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="G49" s="11"/>
+      <c r="H49" s="11"/>
+      <c r="I49" s="11"/>
       <c r="J49" s="3"/>
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
       <c r="N49" s="3"/>
       <c r="O49" s="3"/>
-      <c r="P49" s="12"/>
-    </row>
-    <row r="50" customFormat="1" spans="1:16">
+      <c r="P49" s="21"/>
+    </row>
+    <row r="50" spans="1:16" customFormat="1">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
-      <c r="D50" s="17">
-        <v>5</v>
-      </c>
-      <c r="E50" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F50" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="G50" s="12"/>
-      <c r="H50" s="12"/>
-      <c r="I50" s="12"/>
+      <c r="D50" s="16">
+        <v>14</v>
+      </c>
+      <c r="E50" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="F50" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="G50" s="11"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
       <c r="J50" s="3"/>
       <c r="K50" s="3"/>
       <c r="L50" s="3"/>
       <c r="M50" s="3"/>
       <c r="N50" s="3"/>
       <c r="O50" s="3"/>
-      <c r="P50" s="12"/>
-    </row>
-    <row r="51" customFormat="1" spans="1:16">
+      <c r="P50" s="21"/>
+    </row>
+    <row r="51" spans="1:16" customFormat="1">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
-      <c r="D51" s="17">
-        <v>6</v>
-      </c>
-      <c r="E51" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F51" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G51" s="12"/>
-      <c r="H51" s="12"/>
-      <c r="I51" s="12"/>
+      <c r="D51" s="16">
+        <v>15</v>
+      </c>
+      <c r="E51" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="F51" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="G51" s="11"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
       <c r="J51" s="3"/>
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3"/>
       <c r="N51" s="3"/>
       <c r="O51" s="3"/>
-      <c r="P51" s="12"/>
-    </row>
-    <row r="52" customFormat="1" spans="1:16">
+      <c r="P51" s="11"/>
+    </row>
+    <row r="52" spans="1:16" customFormat="1">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
-      <c r="D52" s="17">
-        <v>7</v>
-      </c>
-      <c r="E52" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F52" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="G52" s="12"/>
-      <c r="H52" s="12"/>
-      <c r="I52" s="12"/>
+      <c r="D52" s="16">
+        <v>16</v>
+      </c>
+      <c r="E52" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="F52" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="G52" s="11"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
       <c r="J52" s="3"/>
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="3"/>
       <c r="N52" s="3"/>
       <c r="O52" s="3"/>
-      <c r="P52" s="12"/>
-    </row>
-    <row r="53" s="1" customFormat="1" spans="1:16">
-      <c r="A53" s="12"/>
-      <c r="B53" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="D53" s="18"/>
-      <c r="E53" s="18"/>
-      <c r="F53" s="19"/>
-      <c r="G53" s="18"/>
-      <c r="H53" s="18"/>
-      <c r="I53" s="18"/>
-      <c r="J53" s="18"/>
-      <c r="K53" s="18"/>
-      <c r="L53" s="18"/>
-      <c r="M53" s="18"/>
-      <c r="N53" s="18"/>
-      <c r="O53" s="18"/>
-      <c r="P53" s="18"/>
-    </row>
-    <row r="54" spans="1:16">
+      <c r="P52" s="11"/>
+    </row>
+    <row r="53" spans="1:16" customFormat="1">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="16">
+        <v>17</v>
+      </c>
+      <c r="E53" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="F53" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+      <c r="J53" s="3"/>
+      <c r="K53" s="3"/>
+      <c r="L53" s="3"/>
+      <c r="M53" s="3"/>
+      <c r="N53" s="3"/>
+      <c r="O53" s="3"/>
+      <c r="P53" s="11"/>
+    </row>
+    <row r="54" spans="1:16" customFormat="1">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="12"/>
-      <c r="F54" s="12"/>
-      <c r="G54" s="12"/>
-      <c r="H54" s="12"/>
-      <c r="I54" s="12"/>
+      <c r="D54" s="16">
+        <v>18</v>
+      </c>
+      <c r="E54" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="F54" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="G54" s="11"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="11"/>
       <c r="J54" s="3"/>
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="3"/>
       <c r="N54" s="3"/>
       <c r="O54" s="3"/>
-      <c r="P54" s="12"/>
-    </row>
-    <row r="55" spans="1:16">
+      <c r="P54" s="11"/>
+    </row>
+    <row r="55" spans="1:16" customFormat="1">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="12"/>
-      <c r="F55" s="12"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="12"/>
-      <c r="I55" s="12"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
       <c r="J55" s="3"/>
       <c r="K55" s="3"/>
       <c r="L55" s="3"/>
       <c r="M55" s="3"/>
       <c r="N55" s="3"/>
       <c r="O55" s="3"/>
-      <c r="P55" s="12"/>
-    </row>
-    <row r="56" s="1" customFormat="1" spans="1:16">
-      <c r="A56" s="12"/>
-      <c r="B56" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C56" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="D56" s="18"/>
-      <c r="E56" s="18"/>
-      <c r="F56" s="12"/>
-      <c r="G56" s="18"/>
-      <c r="H56" s="18"/>
-      <c r="I56" s="18"/>
-      <c r="J56" s="18"/>
-      <c r="K56" s="18"/>
-      <c r="L56" s="18"/>
-      <c r="M56" s="18"/>
-      <c r="N56" s="18"/>
-      <c r="O56" s="18"/>
-      <c r="P56" s="18"/>
-    </row>
-    <row r="57" spans="1:16">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
+      <c r="P55" s="11"/>
+    </row>
+    <row r="56" spans="1:16" customFormat="1">
+      <c r="A56" s="3"/>
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+      <c r="J56" s="3"/>
+      <c r="K56" s="3"/>
+      <c r="L56" s="3"/>
+      <c r="M56" s="3"/>
+      <c r="N56" s="3"/>
+      <c r="O56" s="3"/>
+      <c r="P56" s="11"/>
+    </row>
+    <row r="57" spans="1:16" s="1" customFormat="1">
+      <c r="A57" s="11"/>
+      <c r="B57" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C57" s="17" t="s">
+        <v>45</v>
+      </c>
       <c r="D57" s="17"/>
-      <c r="E57" s="12"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="12"/>
-      <c r="H57" s="12"/>
-      <c r="I57" s="12"/>
-      <c r="J57" s="3"/>
-      <c r="K57" s="3"/>
-      <c r="L57" s="3"/>
-      <c r="M57" s="3"/>
-      <c r="N57" s="3"/>
-      <c r="O57" s="3"/>
-      <c r="P57" s="12"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="17"/>
+      <c r="H57" s="17"/>
+      <c r="I57" s="17"/>
+      <c r="J57" s="17"/>
+      <c r="K57" s="17"/>
+      <c r="L57" s="17"/>
+      <c r="M57" s="17"/>
+      <c r="N57" s="17"/>
+      <c r="O57" s="17"/>
+      <c r="P57" s="17"/>
     </row>
     <row r="58" spans="1:16">
       <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="17"/>
-      <c r="E58" s="12"/>
-      <c r="F58" s="12"/>
-      <c r="G58" s="12"/>
-      <c r="H58" s="12"/>
-      <c r="I58" s="12"/>
+      <c r="B58" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D58" s="16"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
       <c r="J58" s="3"/>
       <c r="K58" s="3"/>
       <c r="L58" s="3"/>
       <c r="M58" s="3"/>
       <c r="N58" s="3"/>
       <c r="O58" s="3"/>
-      <c r="P58" s="12"/>
-    </row>
-    <row r="59" s="1" customFormat="1" spans="1:16">
-      <c r="A59" s="12"/>
-      <c r="B59" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="C59" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="18"/>
-      <c r="G59" s="18"/>
-      <c r="H59" s="18"/>
-      <c r="I59" s="18"/>
-      <c r="J59" s="18"/>
-      <c r="K59" s="18"/>
-      <c r="L59" s="18"/>
-      <c r="M59" s="18"/>
-      <c r="N59" s="18"/>
-      <c r="O59" s="18"/>
-      <c r="P59" s="18"/>
-    </row>
-    <row r="60" spans="1:16">
+      <c r="P58" s="11"/>
+    </row>
+    <row r="59" spans="1:16" customFormat="1">
+      <c r="A59" s="3"/>
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="16">
+        <v>1</v>
+      </c>
+      <c r="E59" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F59" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="3"/>
+      <c r="K59" s="3"/>
+      <c r="L59" s="3"/>
+      <c r="M59" s="3"/>
+      <c r="N59" s="3"/>
+      <c r="O59" s="3"/>
+      <c r="P59" s="11"/>
+    </row>
+    <row r="60" spans="1:16" customFormat="1">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
-      <c r="D60" s="17"/>
-      <c r="E60" s="12"/>
-      <c r="F60" s="12"/>
-      <c r="G60" s="12"/>
-      <c r="H60" s="12"/>
-      <c r="I60" s="12"/>
+      <c r="D60" s="16">
+        <v>2</v>
+      </c>
+      <c r="E60" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F60" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
       <c r="J60" s="3"/>
       <c r="K60" s="3"/>
       <c r="L60" s="3"/>
       <c r="M60" s="3"/>
       <c r="N60" s="3"/>
       <c r="O60" s="3"/>
-      <c r="P60" s="12"/>
-    </row>
-    <row r="61" spans="1:16">
+      <c r="P60" s="11"/>
+    </row>
+    <row r="61" spans="1:16" customFormat="1">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="12"/>
-      <c r="F61" s="12"/>
-      <c r="G61" s="12"/>
-      <c r="H61" s="12"/>
-      <c r="I61" s="12"/>
+      <c r="D61" s="16">
+        <v>3</v>
+      </c>
+      <c r="E61" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F61" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="G61" s="11"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
       <c r="J61" s="3"/>
       <c r="K61" s="3"/>
       <c r="L61" s="3"/>
       <c r="M61" s="3"/>
       <c r="N61" s="3"/>
       <c r="O61" s="3"/>
-      <c r="P61" s="12"/>
-    </row>
-    <row r="62" spans="1:16">
+      <c r="P61" s="11"/>
+    </row>
+    <row r="62" spans="1:16" customFormat="1">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
-      <c r="F62" s="18"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="3"/>
-      <c r="I62" s="3"/>
+      <c r="D62" s="16">
+        <v>4</v>
+      </c>
+      <c r="E62" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="F62" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="G62" s="11"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
       <c r="J62" s="3"/>
       <c r="K62" s="3"/>
       <c r="L62" s="3"/>
       <c r="M62" s="3"/>
       <c r="N62" s="3"/>
       <c r="O62" s="3"/>
-      <c r="P62" s="3"/>
-    </row>
-    <row r="63" spans="1:16">
+      <c r="P62" s="11"/>
+    </row>
+    <row r="63" spans="1:16" customFormat="1">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="E63" s="3"/>
-      <c r="F63" s="12"/>
-      <c r="G63" s="3"/>
-      <c r="H63" s="3"/>
-      <c r="I63" s="3"/>
+      <c r="D63" s="16">
+        <v>5</v>
+      </c>
+      <c r="E63" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="F63" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="G63" s="11"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
       <c r="J63" s="3"/>
       <c r="K63" s="3"/>
       <c r="L63" s="3"/>
       <c r="M63" s="3"/>
       <c r="N63" s="3"/>
       <c r="O63" s="3"/>
-      <c r="P63" s="3"/>
-    </row>
-    <row r="64" spans="1:16">
+      <c r="P63" s="11"/>
+    </row>
+    <row r="64" spans="1:16" customFormat="1">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="12"/>
-      <c r="G64" s="3"/>
-      <c r="H64" s="3"/>
-      <c r="I64" s="3"/>
+      <c r="D64" s="16">
+        <v>6</v>
+      </c>
+      <c r="E64" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="F64" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="G64" s="11"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
       <c r="J64" s="3"/>
       <c r="K64" s="3"/>
       <c r="L64" s="3"/>
       <c r="M64" s="3"/>
       <c r="N64" s="3"/>
       <c r="O64" s="3"/>
-      <c r="P64" s="3"/>
-    </row>
-    <row r="65" spans="1:16">
+      <c r="P64" s="11"/>
+    </row>
+    <row r="65" spans="1:16" customFormat="1">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
-      <c r="D65" s="3"/>
-      <c r="E65" s="3"/>
-      <c r="F65" s="18"/>
-      <c r="G65" s="3"/>
-      <c r="H65" s="3"/>
-      <c r="I65" s="3"/>
+      <c r="D65" s="16"/>
+      <c r="E65" s="11"/>
+      <c r="F65" s="11"/>
+      <c r="G65" s="11"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="11"/>
       <c r="J65" s="3"/>
       <c r="K65" s="3"/>
       <c r="L65" s="3"/>
       <c r="M65" s="3"/>
       <c r="N65" s="3"/>
       <c r="O65" s="3"/>
-      <c r="P65" s="3"/>
-    </row>
-    <row r="66" spans="1:16">
+      <c r="P65" s="11"/>
+    </row>
+    <row r="66" spans="1:16" customFormat="1">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="3"/>
-      <c r="F66" s="12"/>
-      <c r="G66" s="3"/>
-      <c r="H66" s="3"/>
-      <c r="I66" s="3"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="11"/>
+      <c r="F66" s="11"/>
+      <c r="G66" s="11"/>
+      <c r="H66" s="11"/>
+      <c r="I66" s="11"/>
       <c r="J66" s="3"/>
       <c r="K66" s="3"/>
       <c r="L66" s="3"/>
       <c r="M66" s="3"/>
       <c r="N66" s="3"/>
       <c r="O66" s="3"/>
-      <c r="P66" s="3"/>
-    </row>
-    <row r="67" spans="1:16">
+      <c r="P66" s="11"/>
+    </row>
+    <row r="67" spans="1:16" customFormat="1">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="12"/>
-      <c r="G67" s="3"/>
-      <c r="H67" s="3"/>
-      <c r="I67" s="3"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="11"/>
+      <c r="G67" s="11"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
       <c r="J67" s="3"/>
       <c r="K67" s="3"/>
       <c r="L67" s="3"/>
       <c r="M67" s="3"/>
       <c r="N67" s="3"/>
       <c r="O67" s="3"/>
-      <c r="P67" s="3"/>
-    </row>
-    <row r="68" spans="1:16">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-      <c r="G68" s="3"/>
-      <c r="H68" s="3"/>
-      <c r="I68" s="3"/>
-      <c r="J68" s="3"/>
-      <c r="K68" s="3"/>
-      <c r="L68" s="3"/>
-      <c r="M68" s="3"/>
-      <c r="N68" s="3"/>
-      <c r="O68" s="3"/>
-      <c r="P68" s="3"/>
+      <c r="P67" s="11"/>
+    </row>
+    <row r="68" spans="1:16" s="1" customFormat="1">
+      <c r="A68" s="11"/>
+      <c r="B68" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C68" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D68" s="17"/>
+      <c r="E68" s="17"/>
+      <c r="F68" s="18"/>
+      <c r="G68" s="17"/>
+      <c r="H68" s="17"/>
+      <c r="I68" s="17"/>
+      <c r="J68" s="17"/>
+      <c r="K68" s="17"/>
+      <c r="L68" s="17"/>
+      <c r="M68" s="17"/>
+      <c r="N68" s="17"/>
+      <c r="O68" s="17"/>
+      <c r="P68" s="17"/>
     </row>
     <row r="69" spans="1:16">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="3"/>
-      <c r="H69" s="3"/>
-      <c r="I69" s="3"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="11"/>
+      <c r="F69" s="11"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
       <c r="J69" s="3"/>
       <c r="K69" s="3"/>
       <c r="L69" s="3"/>
       <c r="M69" s="3"/>
       <c r="N69" s="3"/>
       <c r="O69" s="3"/>
-      <c r="P69" s="3"/>
+      <c r="P69" s="11"/>
     </row>
     <row r="70" spans="1:16">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
-      <c r="D70" s="3"/>
-      <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="3"/>
-      <c r="H70" s="3"/>
-      <c r="I70" s="3"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="11"/>
+      <c r="F70" s="11"/>
+      <c r="G70" s="11"/>
+      <c r="H70" s="11"/>
+      <c r="I70" s="11"/>
       <c r="J70" s="3"/>
       <c r="K70" s="3"/>
       <c r="L70" s="3"/>
       <c r="M70" s="3"/>
       <c r="N70" s="3"/>
       <c r="O70" s="3"/>
-      <c r="P70" s="3"/>
-    </row>
-    <row r="71" spans="1:16">
-      <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="3"/>
-      <c r="H71" s="3"/>
-      <c r="I71" s="3"/>
-      <c r="J71" s="3"/>
-      <c r="K71" s="3"/>
-      <c r="L71" s="3"/>
-      <c r="M71" s="3"/>
-      <c r="N71" s="3"/>
-      <c r="O71" s="3"/>
-      <c r="P71" s="3"/>
+      <c r="P70" s="11"/>
+    </row>
+    <row r="71" spans="1:16" s="1" customFormat="1">
+      <c r="A71" s="11"/>
+      <c r="B71" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C71" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D71" s="17"/>
+      <c r="E71" s="17"/>
+      <c r="F71" s="11"/>
+      <c r="G71" s="17"/>
+      <c r="H71" s="17"/>
+      <c r="I71" s="17"/>
+      <c r="J71" s="17"/>
+      <c r="K71" s="17"/>
+      <c r="L71" s="17"/>
+      <c r="M71" s="17"/>
+      <c r="N71" s="17"/>
+      <c r="O71" s="17"/>
+      <c r="P71" s="17"/>
     </row>
     <row r="72" spans="1:16">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="3"/>
-      <c r="I72" s="3"/>
+      <c r="D72" s="16"/>
+      <c r="E72" s="11"/>
+      <c r="F72" s="11"/>
+      <c r="G72" s="11"/>
+      <c r="H72" s="11"/>
+      <c r="I72" s="11"/>
       <c r="J72" s="3"/>
       <c r="K72" s="3"/>
       <c r="L72" s="3"/>
       <c r="M72" s="3"/>
       <c r="N72" s="3"/>
       <c r="O72" s="3"/>
-      <c r="P72" s="3"/>
-    </row>
-    <row r="73" spans="3:6">
+      <c r="P72" s="11"/>
+    </row>
+    <row r="73" spans="1:16">
+      <c r="A73" s="3"/>
+      <c r="B73" s="3"/>
       <c r="C73" s="3"/>
-      <c r="F73" s="3"/>
-    </row>
-    <row r="74" spans="3:6">
-      <c r="C74" s="3"/>
-      <c r="F74" s="3"/>
-    </row>
-    <row r="75" spans="3:6">
+      <c r="D73" s="16"/>
+      <c r="E73" s="11"/>
+      <c r="F73" s="11"/>
+      <c r="G73" s="11"/>
+      <c r="H73" s="11"/>
+      <c r="I73" s="11"/>
+      <c r="J73" s="3"/>
+      <c r="K73" s="3"/>
+      <c r="L73" s="3"/>
+      <c r="M73" s="3"/>
+      <c r="N73" s="3"/>
+      <c r="O73" s="3"/>
+      <c r="P73" s="11"/>
+    </row>
+    <row r="74" spans="1:16" s="1" customFormat="1">
+      <c r="A74" s="11"/>
+      <c r="B74" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C74" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D74" s="17"/>
+      <c r="E74" s="17"/>
+      <c r="F74" s="17"/>
+      <c r="G74" s="17"/>
+      <c r="H74" s="17"/>
+      <c r="I74" s="17"/>
+      <c r="J74" s="17"/>
+      <c r="K74" s="17"/>
+      <c r="L74" s="17"/>
+      <c r="M74" s="17"/>
+      <c r="N74" s="17"/>
+      <c r="O74" s="17"/>
+      <c r="P74" s="17"/>
+    </row>
+    <row r="75" spans="1:16">
+      <c r="A75" s="3"/>
+      <c r="B75" s="3"/>
       <c r="C75" s="3"/>
-      <c r="F75" s="3"/>
-    </row>
-    <row r="76" spans="3:6">
+      <c r="D75" s="16"/>
+      <c r="E75" s="11"/>
+      <c r="F75" s="11"/>
+      <c r="G75" s="11"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
+      <c r="J75" s="3"/>
+      <c r="K75" s="3"/>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3"/>
+      <c r="O75" s="3"/>
+      <c r="P75" s="11"/>
+    </row>
+    <row r="76" spans="1:16">
+      <c r="A76" s="3"/>
+      <c r="B76" s="3"/>
       <c r="C76" s="3"/>
-      <c r="F76" s="3"/>
-    </row>
-    <row r="77" spans="3:6">
+      <c r="D76" s="16"/>
+      <c r="E76" s="11"/>
+      <c r="F76" s="11"/>
+      <c r="G76" s="11"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
+      <c r="J76" s="3"/>
+      <c r="K76" s="3"/>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3"/>
+      <c r="N76" s="3"/>
+      <c r="O76" s="3"/>
+      <c r="P76" s="11"/>
+    </row>
+    <row r="77" spans="1:16">
+      <c r="A77" s="3"/>
+      <c r="B77" s="3"/>
       <c r="C77" s="3"/>
-      <c r="F77" s="3"/>
-    </row>
-    <row r="78" spans="3:6">
+      <c r="D77" s="3"/>
+      <c r="E77" s="3"/>
+      <c r="F77" s="17"/>
+      <c r="G77" s="3"/>
+      <c r="H77" s="3"/>
+      <c r="I77" s="3"/>
+      <c r="J77" s="3"/>
+      <c r="K77" s="3"/>
+      <c r="L77" s="3"/>
+      <c r="M77" s="3"/>
+      <c r="N77" s="3"/>
+      <c r="O77" s="3"/>
+      <c r="P77" s="3"/>
+    </row>
+    <row r="78" spans="1:16">
+      <c r="A78" s="3"/>
+      <c r="B78" s="3"/>
       <c r="C78" s="3"/>
-      <c r="F78" s="3"/>
-    </row>
-    <row r="79" spans="3:3">
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="11"/>
+      <c r="G78" s="3"/>
+      <c r="H78" s="3"/>
+      <c r="I78" s="3"/>
+      <c r="J78" s="3"/>
+      <c r="K78" s="3"/>
+      <c r="L78" s="3"/>
+      <c r="M78" s="3"/>
+      <c r="N78" s="3"/>
+      <c r="O78" s="3"/>
+      <c r="P78" s="3"/>
+    </row>
+    <row r="79" spans="1:16">
+      <c r="A79" s="3"/>
+      <c r="B79" s="3"/>
       <c r="C79" s="3"/>
-    </row>
-    <row r="80" spans="3:3">
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="11"/>
+      <c r="G79" s="3"/>
+      <c r="H79" s="3"/>
+      <c r="I79" s="3"/>
+      <c r="J79" s="3"/>
+      <c r="K79" s="3"/>
+      <c r="L79" s="3"/>
+      <c r="M79" s="3"/>
+      <c r="N79" s="3"/>
+      <c r="O79" s="3"/>
+      <c r="P79" s="3"/>
+    </row>
+    <row r="80" spans="1:16">
+      <c r="A80" s="3"/>
+      <c r="B80" s="3"/>
       <c r="C80" s="3"/>
-    </row>
-    <row r="81" spans="3:3">
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="17"/>
+      <c r="G80" s="3"/>
+      <c r="H80" s="3"/>
+      <c r="I80" s="3"/>
+      <c r="J80" s="3"/>
+      <c r="K80" s="3"/>
+      <c r="L80" s="3"/>
+      <c r="M80" s="3"/>
+      <c r="N80" s="3"/>
+      <c r="O80" s="3"/>
+      <c r="P80" s="3"/>
+    </row>
+    <row r="81" spans="1:16">
+      <c r="A81" s="3"/>
+      <c r="B81" s="3"/>
       <c r="C81" s="3"/>
-    </row>
-    <row r="82" spans="3:3">
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+      <c r="F81" s="11"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="3"/>
+      <c r="J81" s="3"/>
+      <c r="K81" s="3"/>
+      <c r="L81" s="3"/>
+      <c r="M81" s="3"/>
+      <c r="N81" s="3"/>
+      <c r="O81" s="3"/>
+      <c r="P81" s="3"/>
+    </row>
+    <row r="82" spans="1:16">
+      <c r="A82" s="3"/>
+      <c r="B82" s="3"/>
       <c r="C82" s="3"/>
-    </row>
-    <row r="83" spans="3:3">
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="11"/>
+      <c r="G82" s="3"/>
+      <c r="H82" s="3"/>
+      <c r="I82" s="3"/>
+      <c r="J82" s="3"/>
+      <c r="K82" s="3"/>
+      <c r="L82" s="3"/>
+      <c r="M82" s="3"/>
+      <c r="N82" s="3"/>
+      <c r="O82" s="3"/>
+      <c r="P82" s="3"/>
+    </row>
+    <row r="83" spans="1:16">
+      <c r="A83" s="3"/>
+      <c r="B83" s="3"/>
       <c r="C83" s="3"/>
-    </row>
-    <row r="84" spans="3:3">
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
+      <c r="H83" s="3"/>
+      <c r="I83" s="3"/>
+      <c r="J83" s="3"/>
+      <c r="K83" s="3"/>
+      <c r="L83" s="3"/>
+      <c r="M83" s="3"/>
+      <c r="N83" s="3"/>
+      <c r="O83" s="3"/>
+      <c r="P83" s="3"/>
+    </row>
+    <row r="84" spans="1:16">
+      <c r="A84" s="3"/>
+      <c r="B84" s="3"/>
       <c r="C84" s="3"/>
-    </row>
-    <row r="85" spans="3:3">
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
+      <c r="I84" s="3"/>
+      <c r="J84" s="3"/>
+      <c r="K84" s="3"/>
+      <c r="L84" s="3"/>
+      <c r="M84" s="3"/>
+      <c r="N84" s="3"/>
+      <c r="O84" s="3"/>
+      <c r="P84" s="3"/>
+    </row>
+    <row r="85" spans="1:16">
+      <c r="A85" s="3"/>
+      <c r="B85" s="3"/>
       <c r="C85" s="3"/>
-    </row>
-    <row r="86" spans="3:3">
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="H85" s="3"/>
+      <c r="I85" s="3"/>
+      <c r="J85" s="3"/>
+      <c r="K85" s="3"/>
+      <c r="L85" s="3"/>
+      <c r="M85" s="3"/>
+      <c r="N85" s="3"/>
+      <c r="O85" s="3"/>
+      <c r="P85" s="3"/>
+    </row>
+    <row r="86" spans="1:16">
+      <c r="A86" s="3"/>
+      <c r="B86" s="3"/>
       <c r="C86" s="3"/>
-    </row>
-    <row r="87" spans="3:3">
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="H86" s="3"/>
+      <c r="I86" s="3"/>
+      <c r="J86" s="3"/>
+      <c r="K86" s="3"/>
+      <c r="L86" s="3"/>
+      <c r="M86" s="3"/>
+      <c r="N86" s="3"/>
+      <c r="O86" s="3"/>
+      <c r="P86" s="3"/>
+    </row>
+    <row r="87" spans="1:16">
+      <c r="A87" s="3"/>
+      <c r="B87" s="3"/>
       <c r="C87" s="3"/>
-    </row>
-    <row r="88" spans="3:3">
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="3"/>
+      <c r="I87" s="3"/>
+      <c r="J87" s="3"/>
+      <c r="K87" s="3"/>
+      <c r="L87" s="3"/>
+      <c r="M87" s="3"/>
+      <c r="N87" s="3"/>
+      <c r="O87" s="3"/>
+      <c r="P87" s="3"/>
+    </row>
+    <row r="88" spans="1:16">
       <c r="C88" s="3"/>
-    </row>
-    <row r="89" spans="3:3">
+      <c r="F88" s="3"/>
+    </row>
+    <row r="89" spans="1:16">
       <c r="C89" s="3"/>
-    </row>
-    <row r="90" spans="3:3">
+      <c r="F89" s="3"/>
+    </row>
+    <row r="90" spans="1:16">
       <c r="C90" s="3"/>
-    </row>
-    <row r="91" spans="3:3">
+      <c r="F90" s="3"/>
+    </row>
+    <row r="91" spans="1:16">
       <c r="C91" s="3"/>
-    </row>
-    <row r="92" spans="3:3">
+      <c r="F91" s="3"/>
+    </row>
+    <row r="92" spans="1:16">
       <c r="C92" s="3"/>
-    </row>
-    <row r="93" spans="3:3">
+      <c r="F92" s="3"/>
+    </row>
+    <row r="93" spans="1:16">
       <c r="C93" s="3"/>
-    </row>
-    <row r="94" spans="3:3">
+      <c r="F93" s="3"/>
+    </row>
+    <row r="94" spans="1:16">
       <c r="C94" s="3"/>
     </row>
-    <row r="95" spans="3:3">
+    <row r="95" spans="1:16">
       <c r="C95" s="3"/>
     </row>
-    <row r="96" spans="3:3">
+    <row r="96" spans="1:16">
       <c r="C96" s="3"/>
     </row>
     <row r="97" spans="3:3">
@@ -5514,34 +5618,78 @@
     <row r="912" spans="3:3">
       <c r="C912" s="3"/>
     </row>
+    <row r="913" spans="3:3">
+      <c r="C913" s="3"/>
+    </row>
+    <row r="914" spans="3:3">
+      <c r="C914" s="3"/>
+    </row>
+    <row r="915" spans="3:3">
+      <c r="C915" s="3"/>
+    </row>
+    <row r="916" spans="3:3">
+      <c r="C916" s="3"/>
+    </row>
+    <row r="917" spans="3:3">
+      <c r="C917" s="3"/>
+    </row>
+    <row r="918" spans="3:3">
+      <c r="C918" s="3"/>
+    </row>
+    <row r="919" spans="3:3">
+      <c r="C919" s="3"/>
+    </row>
+    <row r="920" spans="3:3">
+      <c r="C920" s="3"/>
+    </row>
+    <row r="921" spans="3:3">
+      <c r="C921" s="3"/>
+    </row>
+    <row r="922" spans="3:3">
+      <c r="C922" s="3"/>
+    </row>
+    <row r="923" spans="3:3">
+      <c r="C923" s="3"/>
+    </row>
+    <row r="924" spans="3:3">
+      <c r="C924" s="3"/>
+    </row>
+    <row r="925" spans="3:3">
+      <c r="C925" s="3"/>
+    </row>
+    <row r="926" spans="3:3">
+      <c r="C926" s="3"/>
+    </row>
+    <row r="927" spans="3:3">
+      <c r="C927" s="3"/>
+    </row>
   </sheetData>
   <sheetProtection formatCells="0" formatRows="0" insertRows="0" insertHyperlinks="0" deleteRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="B10:P61">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="B10:P76"/>
   <mergeCells count="1">
     <mergeCell ref="F1:P6"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation allowBlank="1" showInputMessage="1" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C44 C53 C56 C59"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Object Code value" error="The Object code value shall be:&#10;VARIABLE&#10;RECORD&#10;ARRAY" sqref="C36 C37 C38 C39 C42 C43 C45 C46 C52 C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C40:C41 C47:C48 C49:C51 C54:C55 C57:C58 C60:C72">
+    <dataValidation allowBlank="1" showInputMessage="1" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C57 C68 C71 C74"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Object Code value" error="The Object code value shall be:_x000a_VARIABLE_x000a_RECORD_x000a_ARRAY" sqref="C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C58:C67 C69:C70 C72:C73 C75:C87 C36:C56">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Category" error="The value for the entry category shall be &#10;M : (mandatory)&#10;O : (optional) &#10;C : (conditional)" sqref="J36 J37 J38 J39 J42 J43 J45 J46 J52 J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J40:J41 J47:J48 J49:J51 J54:J55 J57:J58 J60:J72">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Category" error="The value for the entry category shall be _x000a_M : (mandatory)_x000a_O : (optional) _x000a_C : (conditional)" sqref="J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J58:J67 J69:J70 J72:J73 J75:J87 J36:J56">
       <formula1>"M,O,C"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Backup/Setting Flag" error="The entry flag shall be&#10;B : (Backup)&#10;S : (Setting)" sqref="K36 K37 K38 K39 K42 K43 K45 K46 K52 K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K40:K41 K47:K48 K49:K51 K54:K55 K57:K58 K60:K72">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Backup/Setting Flag" error="The entry flag shall be_x000a_B : (Backup)_x000a_S : (Setting)" sqref="K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K58:K67 K69:K70 K72:K73 K75:K87 K36:K56">
       <formula1>"B,S"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M36:O36 M37:O37 M38:O38 M39:O39 M42:O42 M43:O43 M45:O45 M46:O46 M52:O52 M12:O13 M18:O19 M24:O25 M30:O31 M40:O41 M54:O55 M60:O61 M15:O16 M21:O22 M27:O28 M33:O34 M47:O48 M57:O58 M49:O51">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M12:O13 M18:O19 M24:O25 M30:O31 M69:O70 M75:O76 M15:O16 M21:O22 M27:O28 M33:O34 M72:O73 M58:O67 M36:O56">
       <formula1>"rx,tx"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C73:C912">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C88:C927">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.236220472440945" right="0.236220472440945" top="0.748031496062992" bottom="0.748031496062992" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" scale="61" fitToWidth="0" fitToHeight="0" orientation="landscape"/>
+  <pageMargins left="0.23622047244094499" right="0.23622047244094499" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" scale="61" fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;L&amp;F&amp;CPage &amp;P of &amp;N</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
1. Add the field "OutF_gantry_velocity_prepare" to xml; 2. Adjust the thread priority;
</commit_message>
<xml_diff>
--- a/ArmCoreV1_QSPI/SSCProject/lan9252_app.xlsx
+++ b/ArmCoreV1_QSPI/SSCProject/lan9252_app.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SI\project\RTM_ON_NEW\FW-ArmCore\ArmCoreV1_QSPI\SSCProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E71522-6154-41A7-B508-5A17479C0666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A209D8DA-B5D9-4902-9B15-B19E1D529420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-7730" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36960" yWindow="-6180" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Profile" sheetId="11" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Profile!$B$10:$P$197</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Profile!$B$1:$P$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Profile!$B$10:$P$198</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Profile!$B$1:$P$199</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="214">
   <si>
     <t>Device Profile:</t>
   </si>
@@ -989,6 +989,13 @@
   <si>
     <t>OutU8_reserved2</t>
     <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>OutF_gantry_velocity_prepare</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>REAL</t>
   </si>
 </sst>
 </file>
@@ -1162,9 +1169,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1175,6 +1179,9 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1481,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T1048"/>
+  <dimension ref="A1:T1049"/>
   <sheetFormatPr defaultColWidth="10.7265625" defaultRowHeight="14" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.81640625" style="2" customWidth="1"/>
@@ -1513,19 +1520,19 @@
         <v>1</v>
       </c>
       <c r="E1" s="4"/>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
       <c r="Q1" s="20"/>
       <c r="R1" s="20"/>
       <c r="S1" s="20"/>
@@ -1541,17 +1548,17 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
       <c r="Q2" s="20"/>
       <c r="R2" s="20"/>
       <c r="S2" s="20"/>
@@ -1563,17 +1570,17 @@
       <c r="C3" s="5"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
       <c r="Q3" s="20"/>
       <c r="R3" s="20"/>
       <c r="S3" s="20"/>
@@ -1585,17 +1592,17 @@
       <c r="C4" s="5"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
       <c r="Q4" s="20"/>
       <c r="R4" s="20"/>
       <c r="S4" s="20"/>
@@ -1607,17 +1614,17 @@
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="26"/>
       <c r="Q5" s="20"/>
       <c r="R5" s="20"/>
       <c r="S5" s="20"/>
@@ -1629,17 +1636,17 @@
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
       <c r="Q6" s="20"/>
       <c r="R6" s="20"/>
       <c r="S6" s="20"/>
@@ -2267,25 +2274,25 @@
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
-      <c r="D37" s="25">
+      <c r="D37" s="24">
         <v>1</v>
       </c>
-      <c r="E37" s="25" t="s">
+      <c r="E37" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F37" s="25" t="s">
+      <c r="F37" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="G37" s="23"/>
-      <c r="H37" s="23"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="24"/>
-      <c r="K37" s="24"/>
-      <c r="L37" s="24"/>
-      <c r="M37" s="24"/>
-      <c r="N37" s="24"/>
-      <c r="O37" s="24"/>
-      <c r="P37" s="22" t="s">
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="I37" s="22"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
+      <c r="M37" s="23"/>
+      <c r="N37" s="23"/>
+      <c r="O37" s="23"/>
+      <c r="P37" s="21" t="s">
         <v>54</v>
       </c>
     </row>
@@ -2293,49 +2300,49 @@
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
-      <c r="D38" s="25">
+      <c r="D38" s="24">
         <v>2</v>
       </c>
-      <c r="E38" s="25" t="s">
+      <c r="E38" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F38" s="25" t="s">
+      <c r="F38" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="G38" s="23"/>
-      <c r="H38" s="23"/>
-      <c r="I38" s="23"/>
-      <c r="J38" s="24"/>
-      <c r="K38" s="24"/>
-      <c r="L38" s="24"/>
-      <c r="M38" s="24"/>
-      <c r="N38" s="24"/>
-      <c r="O38" s="24"/>
-      <c r="P38" s="22"/>
+      <c r="G38" s="22"/>
+      <c r="H38" s="22"/>
+      <c r="I38" s="22"/>
+      <c r="J38" s="23"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="23"/>
+      <c r="M38" s="23"/>
+      <c r="N38" s="23"/>
+      <c r="O38" s="23"/>
+      <c r="P38" s="21"/>
     </row>
     <row r="39" spans="1:16" customFormat="1" ht="14.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
-      <c r="D39" s="25">
+      <c r="D39" s="24">
         <v>3</v>
       </c>
-      <c r="E39" s="25" t="s">
+      <c r="E39" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F39" s="25" t="s">
+      <c r="F39" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="G39" s="23"/>
-      <c r="H39" s="23"/>
-      <c r="I39" s="23"/>
-      <c r="J39" s="24"/>
-      <c r="K39" s="24"/>
-      <c r="L39" s="24"/>
-      <c r="M39" s="24"/>
-      <c r="N39" s="24"/>
-      <c r="O39" s="24"/>
-      <c r="P39" s="22" t="s">
+      <c r="G39" s="22"/>
+      <c r="H39" s="22"/>
+      <c r="I39" s="22"/>
+      <c r="J39" s="23"/>
+      <c r="K39" s="23"/>
+      <c r="L39" s="23"/>
+      <c r="M39" s="23"/>
+      <c r="N39" s="23"/>
+      <c r="O39" s="23"/>
+      <c r="P39" s="21" t="s">
         <v>56</v>
       </c>
     </row>
@@ -2343,13 +2350,13 @@
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
-      <c r="D40" s="25">
+      <c r="D40" s="24">
         <v>4</v>
       </c>
-      <c r="E40" s="25" t="s">
+      <c r="E40" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F40" s="25" t="s">
+      <c r="F40" s="24" t="s">
         <v>63</v>
       </c>
       <c r="G40" s="11"/>
@@ -2369,13 +2376,13 @@
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
-      <c r="D41" s="25">
+      <c r="D41" s="24">
         <v>5</v>
       </c>
-      <c r="E41" s="25" t="s">
+      <c r="E41" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F41" s="25" t="s">
+      <c r="F41" s="24" t="s">
         <v>192</v>
       </c>
       <c r="G41" s="11"/>
@@ -2393,13 +2400,13 @@
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
-      <c r="D42" s="25">
+      <c r="D42" s="24">
         <v>6</v>
       </c>
-      <c r="E42" s="25" t="s">
+      <c r="E42" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F42" s="25" t="s">
+      <c r="F42" s="24" t="s">
         <v>64</v>
       </c>
       <c r="G42" s="11"/>
@@ -2417,13 +2424,13 @@
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
-      <c r="D43" s="25">
+      <c r="D43" s="24">
         <v>7</v>
       </c>
-      <c r="E43" s="25" t="s">
+      <c r="E43" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F43" s="25" t="s">
+      <c r="F43" s="24" t="s">
         <v>65</v>
       </c>
       <c r="G43" s="11"/>
@@ -2441,13 +2448,13 @@
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
-      <c r="D44" s="25">
+      <c r="D44" s="24">
         <v>8</v>
       </c>
-      <c r="E44" s="25" t="s">
+      <c r="E44" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F44" s="25" t="s">
+      <c r="F44" s="24" t="s">
         <v>66</v>
       </c>
       <c r="G44" s="11"/>
@@ -2465,13 +2472,13 @@
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
-      <c r="D45" s="25">
+      <c r="D45" s="24">
         <v>9</v>
       </c>
-      <c r="E45" s="25" t="s">
+      <c r="E45" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F45" s="25" t="s">
+      <c r="F45" s="24" t="s">
         <v>193</v>
       </c>
       <c r="G45" s="11"/>
@@ -2489,13 +2496,13 @@
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
-      <c r="D46" s="25">
+      <c r="D46" s="24">
         <v>10</v>
       </c>
-      <c r="E46" s="25" t="s">
+      <c r="E46" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F46" s="25" t="s">
+      <c r="F46" s="24" t="s">
         <v>67</v>
       </c>
       <c r="G46" s="11"/>
@@ -2513,13 +2520,13 @@
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
-      <c r="D47" s="25">
+      <c r="D47" s="24">
         <v>11</v>
       </c>
-      <c r="E47" s="25" t="s">
+      <c r="E47" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F47" s="25" t="s">
+      <c r="F47" s="24" t="s">
         <v>194</v>
       </c>
       <c r="G47" s="11"/>
@@ -2537,13 +2544,13 @@
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
-      <c r="D48" s="25">
+      <c r="D48" s="24">
         <v>12</v>
       </c>
-      <c r="E48" s="25" t="s">
+      <c r="E48" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F48" s="25" t="s">
+      <c r="F48" s="24" t="s">
         <v>68</v>
       </c>
       <c r="G48" s="11"/>
@@ -2561,13 +2568,13 @@
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
-      <c r="D49" s="25">
+      <c r="D49" s="24">
         <v>13</v>
       </c>
-      <c r="E49" s="25" t="s">
+      <c r="E49" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F49" s="25" t="s">
+      <c r="F49" s="24" t="s">
         <v>69</v>
       </c>
       <c r="G49" s="11"/>
@@ -2585,13 +2592,13 @@
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
-      <c r="D50" s="25">
+      <c r="D50" s="24">
         <v>14</v>
       </c>
-      <c r="E50" s="25" t="s">
+      <c r="E50" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F50" s="25" t="s">
+      <c r="F50" s="24" t="s">
         <v>70</v>
       </c>
       <c r="G50" s="11"/>
@@ -2609,13 +2616,13 @@
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
-      <c r="D51" s="25">
+      <c r="D51" s="24">
         <v>15</v>
       </c>
-      <c r="E51" s="25" t="s">
+      <c r="E51" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F51" s="25" t="s">
+      <c r="F51" s="24" t="s">
         <v>71</v>
       </c>
       <c r="G51" s="11"/>
@@ -2633,13 +2640,13 @@
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
-      <c r="D52" s="25">
+      <c r="D52" s="24">
         <v>16</v>
       </c>
-      <c r="E52" s="25" t="s">
+      <c r="E52" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F52" s="25" t="s">
+      <c r="F52" s="24" t="s">
         <v>72</v>
       </c>
       <c r="G52" s="11"/>
@@ -2657,13 +2664,13 @@
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
-      <c r="D53" s="25">
+      <c r="D53" s="24">
         <v>17</v>
       </c>
-      <c r="E53" s="25" t="s">
+      <c r="E53" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F53" s="25" t="s">
+      <c r="F53" s="24" t="s">
         <v>73</v>
       </c>
       <c r="G53" s="11"/>
@@ -2681,13 +2688,13 @@
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
-      <c r="D54" s="25">
+      <c r="D54" s="24">
         <v>18</v>
       </c>
-      <c r="E54" s="25" t="s">
+      <c r="E54" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F54" s="25" t="s">
+      <c r="F54" s="24" t="s">
         <v>74</v>
       </c>
       <c r="G54" s="11"/>
@@ -2705,13 +2712,13 @@
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
-      <c r="D55" s="25">
+      <c r="D55" s="24">
         <v>19</v>
       </c>
-      <c r="E55" s="25" t="s">
+      <c r="E55" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F55" s="25" t="s">
+      <c r="F55" s="24" t="s">
         <v>195</v>
       </c>
       <c r="G55" s="11"/>
@@ -2729,13 +2736,13 @@
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
-      <c r="D56" s="25">
+      <c r="D56" s="24">
         <v>20</v>
       </c>
-      <c r="E56" s="25" t="s">
+      <c r="E56" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F56" s="25" t="s">
+      <c r="F56" s="24" t="s">
         <v>75</v>
       </c>
       <c r="G56" s="11"/>
@@ -2753,13 +2760,13 @@
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
-      <c r="D57" s="25">
+      <c r="D57" s="24">
         <v>21</v>
       </c>
-      <c r="E57" s="25" t="s">
+      <c r="E57" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F57" s="25" t="s">
+      <c r="F57" s="24" t="s">
         <v>196</v>
       </c>
       <c r="G57" s="11"/>
@@ -2777,13 +2784,13 @@
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
-      <c r="D58" s="25">
+      <c r="D58" s="24">
         <v>22</v>
       </c>
-      <c r="E58" s="25" t="s">
+      <c r="E58" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F58" s="25" t="s">
+      <c r="F58" s="24" t="s">
         <v>76</v>
       </c>
       <c r="G58" s="11"/>
@@ -2801,13 +2808,13 @@
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
-      <c r="D59" s="25">
+      <c r="D59" s="24">
         <v>23</v>
       </c>
-      <c r="E59" s="25" t="s">
+      <c r="E59" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F59" s="25" t="s">
+      <c r="F59" s="24" t="s">
         <v>77</v>
       </c>
       <c r="G59" s="11"/>
@@ -2825,13 +2832,13 @@
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
-      <c r="D60" s="25">
+      <c r="D60" s="24">
         <v>24</v>
       </c>
-      <c r="E60" s="25" t="s">
+      <c r="E60" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F60" s="25" t="s">
+      <c r="F60" s="24" t="s">
         <v>78</v>
       </c>
       <c r="G60" s="11"/>
@@ -2849,13 +2856,13 @@
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
-      <c r="D61" s="25">
+      <c r="D61" s="24">
         <v>25</v>
       </c>
-      <c r="E61" s="25" t="s">
+      <c r="E61" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F61" s="25" t="s">
+      <c r="F61" s="24" t="s">
         <v>79</v>
       </c>
       <c r="G61" s="11"/>
@@ -2873,13 +2880,13 @@
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
-      <c r="D62" s="25">
+      <c r="D62" s="24">
         <v>26</v>
       </c>
-      <c r="E62" s="25" t="s">
+      <c r="E62" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F62" s="25" t="s">
+      <c r="F62" s="24" t="s">
         <v>80</v>
       </c>
       <c r="G62" s="11"/>
@@ -2897,13 +2904,13 @@
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
-      <c r="D63" s="25">
+      <c r="D63" s="24">
         <v>27</v>
       </c>
-      <c r="E63" s="26" t="s">
+      <c r="E63" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="F63" s="26" t="s">
+      <c r="F63" s="25" t="s">
         <v>81</v>
       </c>
       <c r="G63" s="11"/>
@@ -2921,13 +2928,13 @@
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
-      <c r="D64" s="25">
+      <c r="D64" s="24">
         <v>28</v>
       </c>
-      <c r="E64" s="26" t="s">
+      <c r="E64" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="F64" s="26" t="s">
+      <c r="F64" s="25" t="s">
         <v>82</v>
       </c>
       <c r="G64" s="11"/>
@@ -2945,13 +2952,13 @@
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
-      <c r="D65" s="25">
+      <c r="D65" s="24">
         <v>29</v>
       </c>
-      <c r="E65" s="25" t="s">
+      <c r="E65" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F65" s="25" t="s">
+      <c r="F65" s="24" t="s">
         <v>197</v>
       </c>
       <c r="G65" s="11"/>
@@ -2969,13 +2976,13 @@
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
-      <c r="D66" s="25">
+      <c r="D66" s="24">
         <v>30</v>
       </c>
-      <c r="E66" s="26" t="s">
+      <c r="E66" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="F66" s="26" t="s">
+      <c r="F66" s="25" t="s">
         <v>83</v>
       </c>
       <c r="G66" s="11"/>
@@ -2993,13 +3000,13 @@
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
-      <c r="D67" s="25">
+      <c r="D67" s="24">
         <v>31</v>
       </c>
-      <c r="E67" s="26" t="s">
+      <c r="E67" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="F67" s="26" t="s">
+      <c r="F67" s="25" t="s">
         <v>198</v>
       </c>
       <c r="G67" s="11"/>
@@ -3017,13 +3024,13 @@
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
-      <c r="D68" s="25">
+      <c r="D68" s="24">
         <v>32</v>
       </c>
-      <c r="E68" s="26" t="s">
+      <c r="E68" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="F68" s="26" t="s">
+      <c r="F68" s="25" t="s">
         <v>84</v>
       </c>
       <c r="G68" s="11"/>
@@ -3041,13 +3048,13 @@
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
-      <c r="D69" s="25">
+      <c r="D69" s="24">
         <v>33</v>
       </c>
-      <c r="E69" s="26" t="s">
+      <c r="E69" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="F69" s="26" t="s">
+      <c r="F69" s="25" t="s">
         <v>85</v>
       </c>
       <c r="G69" s="11"/>
@@ -3065,13 +3072,13 @@
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
-      <c r="D70" s="25">
+      <c r="D70" s="24">
         <v>34</v>
       </c>
-      <c r="E70" s="26" t="s">
+      <c r="E70" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="F70" s="26" t="s">
+      <c r="F70" s="25" t="s">
         <v>86</v>
       </c>
       <c r="G70" s="11"/>
@@ -3089,13 +3096,13 @@
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
-      <c r="D71" s="25">
+      <c r="D71" s="24">
         <v>35</v>
       </c>
-      <c r="E71" s="26" t="s">
+      <c r="E71" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="F71" s="26" t="s">
+      <c r="F71" s="25" t="s">
         <v>87</v>
       </c>
       <c r="G71" s="11"/>
@@ -3113,13 +3120,13 @@
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
-      <c r="D72" s="25">
+      <c r="D72" s="24">
         <v>36</v>
       </c>
-      <c r="E72" s="26" t="s">
+      <c r="E72" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="F72" s="26" t="s">
+      <c r="F72" s="25" t="s">
         <v>88</v>
       </c>
       <c r="G72" s="11"/>
@@ -3137,13 +3144,13 @@
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
-      <c r="D73" s="25">
+      <c r="D73" s="24">
         <v>37</v>
       </c>
-      <c r="E73" s="25" t="s">
+      <c r="E73" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F73" s="26" t="s">
+      <c r="F73" s="25" t="s">
         <v>90</v>
       </c>
       <c r="G73" s="11"/>
@@ -3161,13 +3168,13 @@
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
-      <c r="D74" s="25">
+      <c r="D74" s="24">
         <v>38</v>
       </c>
-      <c r="E74" s="25" t="s">
+      <c r="E74" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F74" s="26" t="s">
+      <c r="F74" s="25" t="s">
         <v>91</v>
       </c>
       <c r="G74" s="11"/>
@@ -3185,13 +3192,13 @@
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
-      <c r="D75" s="25">
+      <c r="D75" s="24">
         <v>39</v>
       </c>
-      <c r="E75" s="25" t="s">
+      <c r="E75" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F75" s="26" t="s">
+      <c r="F75" s="25" t="s">
         <v>92</v>
       </c>
       <c r="G75" s="11"/>
@@ -3209,13 +3216,13 @@
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
-      <c r="D76" s="25">
+      <c r="D76" s="24">
         <v>40</v>
       </c>
-      <c r="E76" s="25" t="s">
+      <c r="E76" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F76" s="26" t="s">
+      <c r="F76" s="25" t="s">
         <v>93</v>
       </c>
       <c r="G76" s="11"/>
@@ -3233,13 +3240,13 @@
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
-      <c r="D77" s="25">
+      <c r="D77" s="24">
         <v>41</v>
       </c>
-      <c r="E77" s="25" t="s">
+      <c r="E77" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F77" s="26" t="s">
+      <c r="F77" s="25" t="s">
         <v>199</v>
       </c>
       <c r="G77" s="11"/>
@@ -3257,13 +3264,13 @@
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
-      <c r="D78" s="25">
+      <c r="D78" s="24">
         <v>42</v>
       </c>
-      <c r="E78" s="25" t="s">
+      <c r="E78" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F78" s="26" t="s">
+      <c r="F78" s="25" t="s">
         <v>94</v>
       </c>
       <c r="G78" s="11"/>
@@ -3281,13 +3288,13 @@
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
-      <c r="D79" s="25">
+      <c r="D79" s="24">
         <v>43</v>
       </c>
-      <c r="E79" s="25" t="s">
+      <c r="E79" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F79" s="26" t="s">
+      <c r="F79" s="25" t="s">
         <v>95</v>
       </c>
       <c r="G79" s="11"/>
@@ -3305,13 +3312,13 @@
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
-      <c r="D80" s="25">
+      <c r="D80" s="24">
         <v>44</v>
       </c>
-      <c r="E80" s="25" t="s">
+      <c r="E80" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F80" s="26" t="s">
+      <c r="F80" s="25" t="s">
         <v>96</v>
       </c>
       <c r="G80" s="11"/>
@@ -3329,13 +3336,13 @@
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
-      <c r="D81" s="25">
+      <c r="D81" s="24">
         <v>45</v>
       </c>
-      <c r="E81" s="25" t="s">
+      <c r="E81" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F81" s="26" t="s">
+      <c r="F81" s="25" t="s">
         <v>97</v>
       </c>
       <c r="G81" s="11"/>
@@ -3353,13 +3360,13 @@
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
-      <c r="D82" s="25">
+      <c r="D82" s="24">
         <v>46</v>
       </c>
-      <c r="E82" s="25" t="s">
+      <c r="E82" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F82" s="26" t="s">
+      <c r="F82" s="25" t="s">
         <v>200</v>
       </c>
       <c r="G82" s="11"/>
@@ -3377,13 +3384,13 @@
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
-      <c r="D83" s="25">
+      <c r="D83" s="24">
         <v>47</v>
       </c>
-      <c r="E83" s="25" t="s">
+      <c r="E83" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F83" s="26" t="s">
+      <c r="F83" s="25" t="s">
         <v>98</v>
       </c>
       <c r="G83" s="11"/>
@@ -3401,13 +3408,13 @@
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
-      <c r="D84" s="25">
+      <c r="D84" s="24">
         <v>48</v>
       </c>
-      <c r="E84" s="25" t="s">
+      <c r="E84" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F84" s="26" t="s">
+      <c r="F84" s="25" t="s">
         <v>99</v>
       </c>
       <c r="G84" s="11"/>
@@ -3425,13 +3432,13 @@
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
-      <c r="D85" s="25">
+      <c r="D85" s="24">
         <v>49</v>
       </c>
-      <c r="E85" s="25" t="s">
+      <c r="E85" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F85" s="26" t="s">
+      <c r="F85" s="25" t="s">
         <v>100</v>
       </c>
       <c r="G85" s="11"/>
@@ -3449,13 +3456,13 @@
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
-      <c r="D86" s="25">
+      <c r="D86" s="24">
         <v>50</v>
       </c>
-      <c r="E86" s="25" t="s">
+      <c r="E86" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F86" s="25" t="s">
+      <c r="F86" s="24" t="s">
         <v>101</v>
       </c>
       <c r="G86" s="11"/>
@@ -3473,13 +3480,13 @@
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
-      <c r="D87" s="25">
+      <c r="D87" s="24">
         <v>51</v>
       </c>
-      <c r="E87" s="25" t="s">
+      <c r="E87" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F87" s="25" t="s">
+      <c r="F87" s="24" t="s">
         <v>102</v>
       </c>
       <c r="G87" s="11"/>
@@ -3497,13 +3504,13 @@
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
-      <c r="D88" s="25">
+      <c r="D88" s="24">
         <v>52</v>
       </c>
-      <c r="E88" s="25" t="s">
+      <c r="E88" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F88" s="25" t="s">
+      <c r="F88" s="24" t="s">
         <v>201</v>
       </c>
       <c r="G88" s="11"/>
@@ -3521,13 +3528,13 @@
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
-      <c r="D89" s="25">
+      <c r="D89" s="24">
         <v>53</v>
       </c>
-      <c r="E89" s="25" t="s">
+      <c r="E89" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F89" s="25" t="s">
+      <c r="F89" s="24" t="s">
         <v>103</v>
       </c>
       <c r="G89" s="11"/>
@@ -3545,13 +3552,13 @@
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
-      <c r="D90" s="25">
+      <c r="D90" s="24">
         <v>54</v>
       </c>
-      <c r="E90" s="25" t="s">
+      <c r="E90" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F90" s="25" t="s">
+      <c r="F90" s="24" t="s">
         <v>202</v>
       </c>
       <c r="G90" s="11"/>
@@ -3569,13 +3576,13 @@
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
-      <c r="D91" s="25">
+      <c r="D91" s="24">
         <v>55</v>
       </c>
-      <c r="E91" s="25" t="s">
+      <c r="E91" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F91" s="25" t="s">
+      <c r="F91" s="24" t="s">
         <v>104</v>
       </c>
       <c r="G91" s="11"/>
@@ -3593,13 +3600,13 @@
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
-      <c r="D92" s="25">
+      <c r="D92" s="24">
         <v>56</v>
       </c>
-      <c r="E92" s="25" t="s">
+      <c r="E92" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F92" s="25" t="s">
+      <c r="F92" s="24" t="s">
         <v>105</v>
       </c>
       <c r="G92" s="11"/>
@@ -3617,13 +3624,13 @@
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
-      <c r="D93" s="25">
+      <c r="D93" s="24">
         <v>57</v>
       </c>
-      <c r="E93" s="25" t="s">
+      <c r="E93" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F93" s="25" t="s">
+      <c r="F93" s="24" t="s">
         <v>106</v>
       </c>
       <c r="G93" s="11"/>
@@ -3641,13 +3648,13 @@
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
-      <c r="D94" s="25">
+      <c r="D94" s="24">
         <v>58</v>
       </c>
-      <c r="E94" s="25" t="s">
+      <c r="E94" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F94" s="25" t="s">
+      <c r="F94" s="24" t="s">
         <v>107</v>
       </c>
       <c r="G94" s="11"/>
@@ -3665,13 +3672,13 @@
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
-      <c r="D95" s="25">
+      <c r="D95" s="24">
         <v>59</v>
       </c>
-      <c r="E95" s="25" t="s">
+      <c r="E95" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F95" s="25" t="s">
+      <c r="F95" s="24" t="s">
         <v>108</v>
       </c>
       <c r="G95" s="11"/>
@@ -3689,13 +3696,13 @@
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
-      <c r="D96" s="25">
+      <c r="D96" s="24">
         <v>60</v>
       </c>
-      <c r="E96" s="25" t="s">
+      <c r="E96" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F96" s="25" t="s">
+      <c r="F96" s="24" t="s">
         <v>109</v>
       </c>
       <c r="G96" s="11"/>
@@ -3713,13 +3720,13 @@
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
-      <c r="D97" s="25">
+      <c r="D97" s="24">
         <v>61</v>
       </c>
-      <c r="E97" s="25" t="s">
+      <c r="E97" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F97" s="25" t="s">
+      <c r="F97" s="24" t="s">
         <v>110</v>
       </c>
       <c r="G97" s="11"/>
@@ -3737,13 +3744,13 @@
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
-      <c r="D98" s="25">
+      <c r="D98" s="24">
         <v>62</v>
       </c>
-      <c r="E98" s="25" t="s">
+      <c r="E98" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F98" s="25" t="s">
+      <c r="F98" s="24" t="s">
         <v>203</v>
       </c>
       <c r="G98" s="11"/>
@@ -3761,13 +3768,13 @@
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
-      <c r="D99" s="25">
+      <c r="D99" s="24">
         <v>63</v>
       </c>
-      <c r="E99" s="25" t="s">
+      <c r="E99" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F99" s="25" t="s">
+      <c r="F99" s="24" t="s">
         <v>111</v>
       </c>
       <c r="G99" s="11"/>
@@ -3785,13 +3792,13 @@
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
-      <c r="D100" s="25">
+      <c r="D100" s="24">
         <v>64</v>
       </c>
-      <c r="E100" s="25" t="s">
+      <c r="E100" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F100" s="25" t="s">
+      <c r="F100" s="24" t="s">
         <v>204</v>
       </c>
       <c r="G100" s="11"/>
@@ -3809,13 +3816,13 @@
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
-      <c r="D101" s="25">
+      <c r="D101" s="24">
         <v>65</v>
       </c>
-      <c r="E101" s="25" t="s">
+      <c r="E101" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F101" s="25" t="s">
+      <c r="F101" s="24" t="s">
         <v>112</v>
       </c>
       <c r="G101" s="11"/>
@@ -3833,13 +3840,13 @@
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
-      <c r="D102" s="25">
+      <c r="D102" s="24">
         <v>66</v>
       </c>
-      <c r="E102" s="25" t="s">
+      <c r="E102" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F102" s="25" t="s">
+      <c r="F102" s="24" t="s">
         <v>113</v>
       </c>
       <c r="G102" s="11"/>
@@ -3857,13 +3864,13 @@
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
-      <c r="D103" s="25">
+      <c r="D103" s="24">
         <v>67</v>
       </c>
-      <c r="E103" s="25" t="s">
+      <c r="E103" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F103" s="25" t="s">
+      <c r="F103" s="24" t="s">
         <v>114</v>
       </c>
       <c r="G103" s="11"/>
@@ -3881,13 +3888,13 @@
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
-      <c r="D104" s="25">
+      <c r="D104" s="24">
         <v>68</v>
       </c>
-      <c r="E104" s="25" t="s">
+      <c r="E104" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F104" s="25" t="s">
+      <c r="F104" s="24" t="s">
         <v>115</v>
       </c>
       <c r="G104" s="11"/>
@@ -3905,13 +3912,13 @@
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
-      <c r="D105" s="25">
+      <c r="D105" s="24">
         <v>69</v>
       </c>
-      <c r="E105" s="25" t="s">
+      <c r="E105" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F105" s="25" t="s">
+      <c r="F105" s="24" t="s">
         <v>116</v>
       </c>
       <c r="G105" s="11"/>
@@ -3929,13 +3936,13 @@
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
-      <c r="D106" s="25">
+      <c r="D106" s="24">
         <v>70</v>
       </c>
-      <c r="E106" s="25" t="s">
+      <c r="E106" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F106" s="25" t="s">
+      <c r="F106" s="24" t="s">
         <v>117</v>
       </c>
       <c r="G106" s="11"/>
@@ -3953,13 +3960,13 @@
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
-      <c r="D107" s="25">
+      <c r="D107" s="24">
         <v>71</v>
       </c>
-      <c r="E107" s="25" t="s">
+      <c r="E107" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F107" s="25" t="s">
+      <c r="F107" s="24" t="s">
         <v>118</v>
       </c>
       <c r="G107" s="11"/>
@@ -3977,13 +3984,13 @@
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
-      <c r="D108" s="25">
+      <c r="D108" s="24">
         <v>72</v>
       </c>
-      <c r="E108" s="25" t="s">
+      <c r="E108" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F108" s="25" t="s">
+      <c r="F108" s="24" t="s">
         <v>205</v>
       </c>
       <c r="G108" s="11"/>
@@ -4001,13 +4008,13 @@
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
-      <c r="D109" s="25">
+      <c r="D109" s="24">
         <v>73</v>
       </c>
-      <c r="E109" s="25" t="s">
+      <c r="E109" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F109" s="25" t="s">
+      <c r="F109" s="24" t="s">
         <v>119</v>
       </c>
       <c r="G109" s="11"/>
@@ -4025,13 +4032,13 @@
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
-      <c r="D110" s="25">
+      <c r="D110" s="24">
         <v>74</v>
       </c>
-      <c r="E110" s="25" t="s">
+      <c r="E110" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F110" s="25" t="s">
+      <c r="F110" s="24" t="s">
         <v>206</v>
       </c>
       <c r="G110" s="11"/>
@@ -4049,13 +4056,13 @@
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
-      <c r="D111" s="25">
+      <c r="D111" s="24">
         <v>75</v>
       </c>
-      <c r="E111" s="25" t="s">
+      <c r="E111" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F111" s="25" t="s">
+      <c r="F111" s="24" t="s">
         <v>120</v>
       </c>
       <c r="G111" s="11"/>
@@ -4073,13 +4080,13 @@
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
-      <c r="D112" s="25">
+      <c r="D112" s="24">
         <v>76</v>
       </c>
-      <c r="E112" s="25" t="s">
+      <c r="E112" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F112" s="25" t="s">
+      <c r="F112" s="24" t="s">
         <v>121</v>
       </c>
       <c r="G112" s="11"/>
@@ -4097,13 +4104,13 @@
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
-      <c r="D113" s="25">
+      <c r="D113" s="24">
         <v>77</v>
       </c>
-      <c r="E113" s="25" t="s">
+      <c r="E113" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F113" s="25" t="s">
+      <c r="F113" s="24" t="s">
         <v>122</v>
       </c>
       <c r="G113" s="11"/>
@@ -4121,13 +4128,13 @@
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
-      <c r="D114" s="25">
+      <c r="D114" s="24">
         <v>78</v>
       </c>
-      <c r="E114" s="25" t="s">
+      <c r="E114" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F114" s="25" t="s">
+      <c r="F114" s="24" t="s">
         <v>123</v>
       </c>
       <c r="G114" s="11"/>
@@ -4145,13 +4152,13 @@
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
-      <c r="D115" s="25">
+      <c r="D115" s="24">
         <v>79</v>
       </c>
-      <c r="E115" s="25" t="s">
+      <c r="E115" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F115" s="25" t="s">
+      <c r="F115" s="24" t="s">
         <v>124</v>
       </c>
       <c r="G115" s="11"/>
@@ -4169,13 +4176,13 @@
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
-      <c r="D116" s="25">
+      <c r="D116" s="24">
         <v>80</v>
       </c>
-      <c r="E116" s="25" t="s">
+      <c r="E116" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F116" s="25" t="s">
+      <c r="F116" s="24" t="s">
         <v>125</v>
       </c>
       <c r="G116" s="11"/>
@@ -4193,13 +4200,13 @@
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
-      <c r="D117" s="25">
+      <c r="D117" s="24">
         <v>81</v>
       </c>
-      <c r="E117" s="25" t="s">
+      <c r="E117" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F117" s="25" t="s">
+      <c r="F117" s="24" t="s">
         <v>126</v>
       </c>
       <c r="G117" s="11"/>
@@ -4217,13 +4224,13 @@
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
-      <c r="D118" s="25">
+      <c r="D118" s="24">
         <v>82</v>
       </c>
-      <c r="E118" s="25" t="s">
+      <c r="E118" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F118" s="25" t="s">
+      <c r="F118" s="24" t="s">
         <v>127</v>
       </c>
       <c r="G118" s="11"/>
@@ -4241,13 +4248,13 @@
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
-      <c r="D119" s="25">
+      <c r="D119" s="24">
         <v>83</v>
       </c>
-      <c r="E119" s="25" t="s">
+      <c r="E119" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F119" s="25" t="s">
+      <c r="F119" s="24" t="s">
         <v>128</v>
       </c>
       <c r="G119" s="11"/>
@@ -4265,13 +4272,13 @@
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
-      <c r="D120" s="25">
+      <c r="D120" s="24">
         <v>84</v>
       </c>
-      <c r="E120" s="25" t="s">
+      <c r="E120" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F120" s="25" t="s">
+      <c r="F120" s="24" t="s">
         <v>129</v>
       </c>
       <c r="G120" s="11"/>
@@ -4289,13 +4296,13 @@
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
-      <c r="D121" s="25">
+      <c r="D121" s="24">
         <v>85</v>
       </c>
-      <c r="E121" s="25" t="s">
+      <c r="E121" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F121" s="25" t="s">
+      <c r="F121" s="24" t="s">
         <v>207</v>
       </c>
       <c r="G121" s="11"/>
@@ -4313,13 +4320,13 @@
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
-      <c r="D122" s="25">
+      <c r="D122" s="24">
         <v>86</v>
       </c>
-      <c r="E122" s="25" t="s">
+      <c r="E122" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F122" s="25" t="s">
+      <c r="F122" s="24" t="s">
         <v>130</v>
       </c>
       <c r="G122" s="11"/>
@@ -4337,13 +4344,13 @@
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
-      <c r="D123" s="25">
+      <c r="D123" s="24">
         <v>87</v>
       </c>
-      <c r="E123" s="25" t="s">
+      <c r="E123" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F123" s="25" t="s">
+      <c r="F123" s="24" t="s">
         <v>208</v>
       </c>
       <c r="G123" s="11"/>
@@ -4361,13 +4368,13 @@
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
-      <c r="D124" s="25">
+      <c r="D124" s="24">
         <v>88</v>
       </c>
-      <c r="E124" s="25" t="s">
+      <c r="E124" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F124" s="25" t="s">
+      <c r="F124" s="24" t="s">
         <v>131</v>
       </c>
       <c r="G124" s="11"/>
@@ -4385,13 +4392,13 @@
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
-      <c r="D125" s="25">
+      <c r="D125" s="24">
         <v>89</v>
       </c>
-      <c r="E125" s="25" t="s">
+      <c r="E125" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F125" s="25" t="s">
+      <c r="F125" s="24" t="s">
         <v>132</v>
       </c>
       <c r="G125" s="11"/>
@@ -4409,13 +4416,13 @@
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
-      <c r="D126" s="25">
+      <c r="D126" s="24">
         <v>90</v>
       </c>
-      <c r="E126" s="25" t="s">
+      <c r="E126" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F126" s="25" t="s">
+      <c r="F126" s="24" t="s">
         <v>133</v>
       </c>
       <c r="G126" s="11"/>
@@ -4433,13 +4440,13 @@
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
-      <c r="D127" s="25">
+      <c r="D127" s="24">
         <v>91</v>
       </c>
-      <c r="E127" s="25" t="s">
+      <c r="E127" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F127" s="25" t="s">
+      <c r="F127" s="24" t="s">
         <v>134</v>
       </c>
       <c r="G127" s="11"/>
@@ -4457,13 +4464,13 @@
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
-      <c r="D128" s="25">
+      <c r="D128" s="24">
         <v>92</v>
       </c>
-      <c r="E128" s="25" t="s">
+      <c r="E128" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F128" s="25" t="s">
+      <c r="F128" s="24" t="s">
         <v>135</v>
       </c>
       <c r="G128" s="11"/>
@@ -4481,13 +4488,13 @@
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
-      <c r="D129" s="25">
+      <c r="D129" s="24">
         <v>93</v>
       </c>
-      <c r="E129" s="25" t="s">
+      <c r="E129" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F129" s="25" t="s">
+      <c r="F129" s="24" t="s">
         <v>136</v>
       </c>
       <c r="G129" s="11"/>
@@ -4505,13 +4512,13 @@
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
-      <c r="D130" s="25">
+      <c r="D130" s="24">
         <v>94</v>
       </c>
-      <c r="E130" s="25" t="s">
+      <c r="E130" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F130" s="25" t="s">
+      <c r="F130" s="24" t="s">
         <v>137</v>
       </c>
       <c r="G130" s="11"/>
@@ -4529,13 +4536,13 @@
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
-      <c r="D131" s="25">
+      <c r="D131" s="24">
         <v>95</v>
       </c>
-      <c r="E131" s="25" t="s">
+      <c r="E131" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F131" s="25" t="s">
+      <c r="F131" s="24" t="s">
         <v>138</v>
       </c>
       <c r="G131" s="11"/>
@@ -4553,13 +4560,13 @@
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
-      <c r="D132" s="25">
+      <c r="D132" s="24">
         <v>96</v>
       </c>
-      <c r="E132" s="25" t="s">
+      <c r="E132" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F132" s="25" t="s">
+      <c r="F132" s="24" t="s">
         <v>139</v>
       </c>
       <c r="G132" s="11"/>
@@ -4577,13 +4584,13 @@
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
-      <c r="D133" s="25">
+      <c r="D133" s="24">
         <v>97</v>
       </c>
-      <c r="E133" s="25" t="s">
+      <c r="E133" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F133" s="25" t="s">
+      <c r="F133" s="24" t="s">
         <v>140</v>
       </c>
       <c r="G133" s="11"/>
@@ -4601,13 +4608,13 @@
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
-      <c r="D134" s="25">
+      <c r="D134" s="24">
         <v>98</v>
       </c>
-      <c r="E134" s="25" t="s">
+      <c r="E134" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F134" s="25" t="s">
+      <c r="F134" s="24" t="s">
         <v>141</v>
       </c>
       <c r="G134" s="11"/>
@@ -4625,13 +4632,13 @@
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
-      <c r="D135" s="25">
+      <c r="D135" s="24">
         <v>99</v>
       </c>
-      <c r="E135" s="25" t="s">
+      <c r="E135" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F135" s="25" t="s">
+      <c r="F135" s="24" t="s">
         <v>142</v>
       </c>
       <c r="G135" s="11"/>
@@ -4649,13 +4656,13 @@
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
-      <c r="D136" s="25">
+      <c r="D136" s="24">
         <v>100</v>
       </c>
-      <c r="E136" s="25" t="s">
+      <c r="E136" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F136" s="25" t="s">
+      <c r="F136" s="24" t="s">
         <v>143</v>
       </c>
       <c r="G136" s="11"/>
@@ -4673,13 +4680,13 @@
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
-      <c r="D137" s="25">
+      <c r="D137" s="24">
         <v>101</v>
       </c>
-      <c r="E137" s="25" t="s">
+      <c r="E137" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F137" s="25" t="s">
+      <c r="F137" s="24" t="s">
         <v>144</v>
       </c>
       <c r="G137" s="11"/>
@@ -4697,13 +4704,13 @@
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
-      <c r="D138" s="25">
+      <c r="D138" s="24">
         <v>102</v>
       </c>
-      <c r="E138" s="25" t="s">
+      <c r="E138" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F138" s="25" t="s">
+      <c r="F138" s="24" t="s">
         <v>145</v>
       </c>
       <c r="G138" s="11"/>
@@ -4721,13 +4728,13 @@
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
-      <c r="D139" s="25">
+      <c r="D139" s="24">
         <v>103</v>
       </c>
-      <c r="E139" s="25" t="s">
+      <c r="E139" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F139" s="25" t="s">
+      <c r="F139" s="24" t="s">
         <v>146</v>
       </c>
       <c r="G139" s="11"/>
@@ -4745,13 +4752,13 @@
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
-      <c r="D140" s="25">
+      <c r="D140" s="24">
         <v>104</v>
       </c>
-      <c r="E140" s="25" t="s">
+      <c r="E140" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F140" s="25" t="s">
+      <c r="F140" s="24" t="s">
         <v>147</v>
       </c>
       <c r="G140" s="11"/>
@@ -4769,13 +4776,13 @@
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
-      <c r="D141" s="25">
+      <c r="D141" s="24">
         <v>105</v>
       </c>
-      <c r="E141" s="25" t="s">
+      <c r="E141" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F141" s="25" t="s">
+      <c r="F141" s="24" t="s">
         <v>148</v>
       </c>
       <c r="G141" s="11"/>
@@ -4793,13 +4800,13 @@
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
-      <c r="D142" s="25">
+      <c r="D142" s="24">
         <v>106</v>
       </c>
-      <c r="E142" s="25" t="s">
+      <c r="E142" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F142" s="25" t="s">
+      <c r="F142" s="24" t="s">
         <v>149</v>
       </c>
       <c r="G142" s="11"/>
@@ -4817,13 +4824,13 @@
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
-      <c r="D143" s="25">
+      <c r="D143" s="24">
         <v>107</v>
       </c>
-      <c r="E143" s="25" t="s">
+      <c r="E143" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F143" s="25" t="s">
+      <c r="F143" s="24" t="s">
         <v>150</v>
       </c>
       <c r="G143" s="11"/>
@@ -4890,10 +4897,10 @@
       <c r="D146" s="16">
         <v>1</v>
       </c>
-      <c r="E146" s="25" t="s">
+      <c r="E146" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F146" s="25" t="s">
+      <c r="F146" s="24" t="s">
         <v>151</v>
       </c>
       <c r="G146" s="11"/>
@@ -4914,10 +4921,10 @@
       <c r="D147" s="16">
         <v>2</v>
       </c>
-      <c r="E147" s="25" t="s">
+      <c r="E147" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F147" s="25" t="s">
+      <c r="F147" s="24" t="s">
         <v>209</v>
       </c>
       <c r="G147" s="11"/>
@@ -4938,10 +4945,10 @@
       <c r="D148" s="16">
         <v>3</v>
       </c>
-      <c r="E148" s="25" t="s">
+      <c r="E148" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F148" s="25" t="s">
+      <c r="F148" s="24" t="s">
         <v>152</v>
       </c>
       <c r="G148" s="11"/>
@@ -4962,10 +4969,10 @@
       <c r="D149" s="16">
         <v>4</v>
       </c>
-      <c r="E149" s="25" t="s">
+      <c r="E149" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F149" s="25" t="s">
+      <c r="F149" s="24" t="s">
         <v>153</v>
       </c>
       <c r="G149" s="11"/>
@@ -4986,10 +4993,10 @@
       <c r="D150" s="16">
         <v>5</v>
       </c>
-      <c r="E150" s="25" t="s">
+      <c r="E150" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F150" s="25" t="s">
+      <c r="F150" s="24" t="s">
         <v>210</v>
       </c>
       <c r="G150" s="11"/>
@@ -5010,10 +5017,10 @@
       <c r="D151" s="16">
         <v>6</v>
       </c>
-      <c r="E151" s="25" t="s">
+      <c r="E151" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F151" s="25" t="s">
+      <c r="F151" s="24" t="s">
         <v>154</v>
       </c>
       <c r="G151" s="11"/>
@@ -5034,10 +5041,10 @@
       <c r="D152" s="16">
         <v>7</v>
       </c>
-      <c r="E152" s="25" t="s">
+      <c r="E152" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F152" s="25" t="s">
+      <c r="F152" s="24" t="s">
         <v>155</v>
       </c>
       <c r="G152" s="11"/>
@@ -5058,10 +5065,10 @@
       <c r="D153" s="16">
         <v>8</v>
       </c>
-      <c r="E153" s="25" t="s">
+      <c r="E153" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F153" s="25" t="s">
+      <c r="F153" s="24" t="s">
         <v>156</v>
       </c>
       <c r="G153" s="11"/>
@@ -5082,10 +5089,10 @@
       <c r="D154" s="16">
         <v>9</v>
       </c>
-      <c r="E154" s="25" t="s">
+      <c r="E154" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F154" s="25" t="s">
+      <c r="F154" s="24" t="s">
         <v>157</v>
       </c>
       <c r="G154" s="11"/>
@@ -5106,10 +5113,10 @@
       <c r="D155" s="16">
         <v>10</v>
       </c>
-      <c r="E155" s="25" t="s">
+      <c r="E155" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F155" s="25" t="s">
+      <c r="F155" s="24" t="s">
         <v>158</v>
       </c>
       <c r="G155" s="11"/>
@@ -5130,10 +5137,10 @@
       <c r="D156" s="16">
         <v>11</v>
       </c>
-      <c r="E156" s="25" t="s">
+      <c r="E156" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F156" s="25" t="s">
+      <c r="F156" s="24" t="s">
         <v>159</v>
       </c>
       <c r="G156" s="11"/>
@@ -5154,10 +5161,10 @@
       <c r="D157" s="16">
         <v>12</v>
       </c>
-      <c r="E157" s="25" t="s">
+      <c r="E157" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F157" s="25" t="s">
+      <c r="F157" s="24" t="s">
         <v>160</v>
       </c>
       <c r="G157" s="11"/>
@@ -5178,10 +5185,10 @@
       <c r="D158" s="16">
         <v>13</v>
       </c>
-      <c r="E158" s="25" t="s">
+      <c r="E158" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F158" s="25" t="s">
+      <c r="F158" s="24" t="s">
         <v>163</v>
       </c>
       <c r="G158" s="11"/>
@@ -5202,11 +5209,11 @@
       <c r="D159" s="16">
         <v>14</v>
       </c>
-      <c r="E159" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F159" s="25" t="s">
-        <v>161</v>
+      <c r="E159" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="F159" s="24" t="s">
+        <v>212</v>
       </c>
       <c r="G159" s="11"/>
       <c r="H159" s="11"/>
@@ -5226,11 +5233,11 @@
       <c r="D160" s="16">
         <v>15</v>
       </c>
-      <c r="E160" s="25" t="s">
+      <c r="E160" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F160" s="25" t="s">
-        <v>162</v>
+      <c r="F160" s="24" t="s">
+        <v>161</v>
       </c>
       <c r="G160" s="11"/>
       <c r="H160" s="11"/>
@@ -5250,11 +5257,11 @@
       <c r="D161" s="16">
         <v>16</v>
       </c>
-      <c r="E161" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F161" s="25" t="s">
-        <v>164</v>
+      <c r="E161" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="F161" s="24" t="s">
+        <v>162</v>
       </c>
       <c r="G161" s="11"/>
       <c r="H161" s="11"/>
@@ -5274,11 +5281,11 @@
       <c r="D162" s="16">
         <v>17</v>
       </c>
-      <c r="E162" s="25" t="s">
+      <c r="E162" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F162" s="25" t="s">
-        <v>165</v>
+      <c r="F162" s="24" t="s">
+        <v>164</v>
       </c>
       <c r="G162" s="11"/>
       <c r="H162" s="11"/>
@@ -5298,11 +5305,11 @@
       <c r="D163" s="16">
         <v>18</v>
       </c>
-      <c r="E163" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F163" s="25" t="s">
-        <v>166</v>
+      <c r="E163" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F163" s="24" t="s">
+        <v>165</v>
       </c>
       <c r="G163" s="11"/>
       <c r="H163" s="11"/>
@@ -5322,11 +5329,11 @@
       <c r="D164" s="16">
         <v>19</v>
       </c>
-      <c r="E164" s="25" t="s">
+      <c r="E164" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F164" s="25" t="s">
-        <v>167</v>
+      <c r="F164" s="24" t="s">
+        <v>166</v>
       </c>
       <c r="G164" s="11"/>
       <c r="H164" s="11"/>
@@ -5346,11 +5353,11 @@
       <c r="D165" s="16">
         <v>20</v>
       </c>
-      <c r="E165" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F165" s="25" t="s">
-        <v>168</v>
+      <c r="E165" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="F165" s="24" t="s">
+        <v>167</v>
       </c>
       <c r="G165" s="11"/>
       <c r="H165" s="11"/>
@@ -5370,11 +5377,11 @@
       <c r="D166" s="16">
         <v>21</v>
       </c>
-      <c r="E166" s="25" t="s">
+      <c r="E166" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F166" s="25" t="s">
-        <v>169</v>
+      <c r="F166" s="24" t="s">
+        <v>168</v>
       </c>
       <c r="G166" s="11"/>
       <c r="H166" s="11"/>
@@ -5394,11 +5401,11 @@
       <c r="D167" s="16">
         <v>22</v>
       </c>
-      <c r="E167" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F167" s="25" t="s">
-        <v>170</v>
+      <c r="E167" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F167" s="24" t="s">
+        <v>169</v>
       </c>
       <c r="G167" s="11"/>
       <c r="H167" s="11"/>
@@ -5418,11 +5425,11 @@
       <c r="D168" s="16">
         <v>23</v>
       </c>
-      <c r="E168" s="25" t="s">
+      <c r="E168" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F168" s="25" t="s">
-        <v>171</v>
+      <c r="F168" s="24" t="s">
+        <v>170</v>
       </c>
       <c r="G168" s="11"/>
       <c r="H168" s="11"/>
@@ -5442,11 +5449,11 @@
       <c r="D169" s="16">
         <v>24</v>
       </c>
-      <c r="E169" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F169" s="25" t="s">
-        <v>172</v>
+      <c r="E169" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="F169" s="24" t="s">
+        <v>171</v>
       </c>
       <c r="G169" s="11"/>
       <c r="H169" s="11"/>
@@ -5466,11 +5473,11 @@
       <c r="D170" s="16">
         <v>25</v>
       </c>
-      <c r="E170" s="25" t="s">
+      <c r="E170" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F170" s="25" t="s">
-        <v>173</v>
+      <c r="F170" s="24" t="s">
+        <v>172</v>
       </c>
       <c r="G170" s="11"/>
       <c r="H170" s="11"/>
@@ -5490,11 +5497,11 @@
       <c r="D171" s="16">
         <v>26</v>
       </c>
-      <c r="E171" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F171" s="25" t="s">
-        <v>174</v>
+      <c r="E171" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F171" s="24" t="s">
+        <v>173</v>
       </c>
       <c r="G171" s="11"/>
       <c r="H171" s="11"/>
@@ -5514,11 +5521,11 @@
       <c r="D172" s="16">
         <v>27</v>
       </c>
-      <c r="E172" s="25" t="s">
+      <c r="E172" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F172" s="25" t="s">
-        <v>175</v>
+      <c r="F172" s="24" t="s">
+        <v>174</v>
       </c>
       <c r="G172" s="11"/>
       <c r="H172" s="11"/>
@@ -5538,11 +5545,11 @@
       <c r="D173" s="16">
         <v>28</v>
       </c>
-      <c r="E173" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F173" s="25" t="s">
-        <v>176</v>
+      <c r="E173" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="F173" s="24" t="s">
+        <v>175</v>
       </c>
       <c r="G173" s="11"/>
       <c r="H173" s="11"/>
@@ -5562,11 +5569,11 @@
       <c r="D174" s="16">
         <v>29</v>
       </c>
-      <c r="E174" s="25" t="s">
+      <c r="E174" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F174" s="25" t="s">
-        <v>177</v>
+      <c r="F174" s="24" t="s">
+        <v>176</v>
       </c>
       <c r="G174" s="11"/>
       <c r="H174" s="11"/>
@@ -5586,11 +5593,11 @@
       <c r="D175" s="16">
         <v>30</v>
       </c>
-      <c r="E175" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F175" s="25" t="s">
-        <v>178</v>
+      <c r="E175" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F175" s="24" t="s">
+        <v>177</v>
       </c>
       <c r="G175" s="11"/>
       <c r="H175" s="11"/>
@@ -5610,11 +5617,11 @@
       <c r="D176" s="16">
         <v>31</v>
       </c>
-      <c r="E176" s="25" t="s">
+      <c r="E176" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F176" s="25" t="s">
-        <v>179</v>
+      <c r="F176" s="24" t="s">
+        <v>178</v>
       </c>
       <c r="G176" s="11"/>
       <c r="H176" s="11"/>
@@ -5634,11 +5641,11 @@
       <c r="D177" s="16">
         <v>32</v>
       </c>
-      <c r="E177" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F177" s="25" t="s">
-        <v>190</v>
+      <c r="E177" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="F177" s="24" t="s">
+        <v>179</v>
       </c>
       <c r="G177" s="11"/>
       <c r="H177" s="11"/>
@@ -5658,11 +5665,11 @@
       <c r="D178" s="16">
         <v>33</v>
       </c>
-      <c r="E178" s="25" t="s">
+      <c r="E178" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F178" s="25" t="s">
-        <v>211</v>
+      <c r="F178" s="24" t="s">
+        <v>190</v>
       </c>
       <c r="G178" s="11"/>
       <c r="H178" s="11"/>
@@ -5682,11 +5689,11 @@
       <c r="D179" s="16">
         <v>34</v>
       </c>
-      <c r="E179" s="25" t="s">
+      <c r="E179" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F179" s="25" t="s">
-        <v>180</v>
+      <c r="F179" s="24" t="s">
+        <v>211</v>
       </c>
       <c r="G179" s="11"/>
       <c r="H179" s="11"/>
@@ -5706,11 +5713,11 @@
       <c r="D180" s="16">
         <v>35</v>
       </c>
-      <c r="E180" s="25" t="s">
+      <c r="E180" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F180" s="25" t="s">
-        <v>181</v>
+      <c r="F180" s="24" t="s">
+        <v>180</v>
       </c>
       <c r="G180" s="11"/>
       <c r="H180" s="11"/>
@@ -5730,11 +5737,11 @@
       <c r="D181" s="16">
         <v>36</v>
       </c>
-      <c r="E181" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F181" s="25" t="s">
-        <v>182</v>
+      <c r="E181" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F181" s="24" t="s">
+        <v>181</v>
       </c>
       <c r="G181" s="11"/>
       <c r="H181" s="11"/>
@@ -5754,11 +5761,11 @@
       <c r="D182" s="16">
         <v>37</v>
       </c>
-      <c r="E182" s="25" t="s">
+      <c r="E182" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F182" s="25" t="s">
-        <v>183</v>
+      <c r="F182" s="24" t="s">
+        <v>182</v>
       </c>
       <c r="G182" s="11"/>
       <c r="H182" s="11"/>
@@ -5778,11 +5785,11 @@
       <c r="D183" s="16">
         <v>38</v>
       </c>
-      <c r="E183" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F183" s="25" t="s">
-        <v>184</v>
+      <c r="E183" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="F183" s="24" t="s">
+        <v>183</v>
       </c>
       <c r="G183" s="11"/>
       <c r="H183" s="11"/>
@@ -5802,11 +5809,11 @@
       <c r="D184" s="16">
         <v>39</v>
       </c>
-      <c r="E184" s="25" t="s">
+      <c r="E184" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F184" s="25" t="s">
-        <v>185</v>
+      <c r="F184" s="24" t="s">
+        <v>184</v>
       </c>
       <c r="G184" s="11"/>
       <c r="H184" s="11"/>
@@ -5826,11 +5833,11 @@
       <c r="D185" s="16">
         <v>40</v>
       </c>
-      <c r="E185" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="F185" s="25" t="s">
-        <v>186</v>
+      <c r="E185" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F185" s="24" t="s">
+        <v>185</v>
       </c>
       <c r="G185" s="11"/>
       <c r="H185" s="11"/>
@@ -5850,11 +5857,11 @@
       <c r="D186" s="16">
         <v>41</v>
       </c>
-      <c r="E186" s="25" t="s">
+      <c r="E186" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="F186" s="25" t="s">
-        <v>187</v>
+      <c r="F186" s="24" t="s">
+        <v>186</v>
       </c>
       <c r="G186" s="11"/>
       <c r="H186" s="11"/>
@@ -5874,11 +5881,11 @@
       <c r="D187" s="16">
         <v>42</v>
       </c>
-      <c r="E187" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="F187" s="25" t="s">
-        <v>188</v>
+      <c r="E187" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="F187" s="24" t="s">
+        <v>187</v>
       </c>
       <c r="G187" s="11"/>
       <c r="H187" s="11"/>
@@ -5898,11 +5905,11 @@
       <c r="D188" s="16">
         <v>43</v>
       </c>
-      <c r="E188" s="25" t="s">
+      <c r="E188" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="F188" s="25" t="s">
-        <v>189</v>
+      <c r="F188" s="24" t="s">
+        <v>188</v>
       </c>
       <c r="G188" s="11"/>
       <c r="H188" s="11"/>
@@ -5915,45 +5922,51 @@
       <c r="O188" s="3"/>
       <c r="P188" s="11"/>
     </row>
-    <row r="189" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A189" s="11"/>
-      <c r="B189" s="17" t="s">
+    <row r="189" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="3"/>
+      <c r="B189" s="3"/>
+      <c r="C189" s="3"/>
+      <c r="D189" s="16">
+        <v>44</v>
+      </c>
+      <c r="E189" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="F189" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="G189" s="11"/>
+      <c r="H189" s="11"/>
+      <c r="I189" s="11"/>
+      <c r="J189" s="3"/>
+      <c r="K189" s="3"/>
+      <c r="L189" s="3"/>
+      <c r="M189" s="3"/>
+      <c r="N189" s="3"/>
+      <c r="O189" s="3"/>
+      <c r="P189" s="11"/>
+    </row>
+    <row r="190" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="11"/>
+      <c r="B190" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C189" s="17" t="s">
+      <c r="C190" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="D189" s="17"/>
-      <c r="E189" s="17"/>
-      <c r="F189" s="18"/>
-      <c r="G189" s="17"/>
-      <c r="H189" s="17"/>
-      <c r="I189" s="17"/>
-      <c r="J189" s="17"/>
-      <c r="K189" s="17"/>
-      <c r="L189" s="17"/>
-      <c r="M189" s="17"/>
-      <c r="N189" s="17"/>
-      <c r="O189" s="17"/>
-      <c r="P189" s="17"/>
-    </row>
-    <row r="190" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A190" s="3"/>
-      <c r="B190" s="3"/>
-      <c r="C190" s="3"/>
-      <c r="D190" s="16"/>
-      <c r="E190" s="11"/>
-      <c r="F190" s="11"/>
-      <c r="G190" s="11"/>
-      <c r="H190" s="11"/>
-      <c r="I190" s="11"/>
-      <c r="J190" s="3"/>
-      <c r="K190" s="3"/>
-      <c r="L190" s="3"/>
-      <c r="M190" s="3"/>
-      <c r="N190" s="3"/>
-      <c r="O190" s="3"/>
-      <c r="P190" s="11"/>
+      <c r="D190" s="17"/>
+      <c r="E190" s="17"/>
+      <c r="F190" s="18"/>
+      <c r="G190" s="17"/>
+      <c r="H190" s="17"/>
+      <c r="I190" s="17"/>
+      <c r="J190" s="17"/>
+      <c r="K190" s="17"/>
+      <c r="L190" s="17"/>
+      <c r="M190" s="17"/>
+      <c r="N190" s="17"/>
+      <c r="O190" s="17"/>
+      <c r="P190" s="17"/>
     </row>
     <row r="191" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A191" s="3"/>
@@ -5973,45 +5986,45 @@
       <c r="O191" s="3"/>
       <c r="P191" s="11"/>
     </row>
-    <row r="192" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A192" s="11"/>
-      <c r="B192" s="17" t="s">
+    <row r="192" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A192" s="3"/>
+      <c r="B192" s="3"/>
+      <c r="C192" s="3"/>
+      <c r="D192" s="16"/>
+      <c r="E192" s="11"/>
+      <c r="F192" s="11"/>
+      <c r="G192" s="11"/>
+      <c r="H192" s="11"/>
+      <c r="I192" s="11"/>
+      <c r="J192" s="3"/>
+      <c r="K192" s="3"/>
+      <c r="L192" s="3"/>
+      <c r="M192" s="3"/>
+      <c r="N192" s="3"/>
+      <c r="O192" s="3"/>
+      <c r="P192" s="11"/>
+    </row>
+    <row r="193" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="11"/>
+      <c r="B193" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="C192" s="17" t="s">
+      <c r="C193" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="D192" s="17"/>
-      <c r="E192" s="17"/>
-      <c r="F192" s="11"/>
-      <c r="G192" s="17"/>
-      <c r="H192" s="17"/>
-      <c r="I192" s="17"/>
-      <c r="J192" s="17"/>
-      <c r="K192" s="17"/>
-      <c r="L192" s="17"/>
-      <c r="M192" s="17"/>
-      <c r="N192" s="17"/>
-      <c r="O192" s="17"/>
-      <c r="P192" s="17"/>
-    </row>
-    <row r="193" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A193" s="3"/>
-      <c r="B193" s="3"/>
-      <c r="C193" s="3"/>
-      <c r="D193" s="16"/>
-      <c r="E193" s="11"/>
+      <c r="D193" s="17"/>
+      <c r="E193" s="17"/>
       <c r="F193" s="11"/>
-      <c r="G193" s="11"/>
-      <c r="H193" s="11"/>
-      <c r="I193" s="11"/>
-      <c r="J193" s="3"/>
-      <c r="K193" s="3"/>
-      <c r="L193" s="3"/>
-      <c r="M193" s="3"/>
-      <c r="N193" s="3"/>
-      <c r="O193" s="3"/>
-      <c r="P193" s="11"/>
+      <c r="G193" s="17"/>
+      <c r="H193" s="17"/>
+      <c r="I193" s="17"/>
+      <c r="J193" s="17"/>
+      <c r="K193" s="17"/>
+      <c r="L193" s="17"/>
+      <c r="M193" s="17"/>
+      <c r="N193" s="17"/>
+      <c r="O193" s="17"/>
+      <c r="P193" s="17"/>
     </row>
     <row r="194" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A194" s="3"/>
@@ -6031,45 +6044,45 @@
       <c r="O194" s="3"/>
       <c r="P194" s="11"/>
     </row>
-    <row r="195" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A195" s="11"/>
-      <c r="B195" s="17" t="s">
+    <row r="195" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A195" s="3"/>
+      <c r="B195" s="3"/>
+      <c r="C195" s="3"/>
+      <c r="D195" s="16"/>
+      <c r="E195" s="11"/>
+      <c r="F195" s="11"/>
+      <c r="G195" s="11"/>
+      <c r="H195" s="11"/>
+      <c r="I195" s="11"/>
+      <c r="J195" s="3"/>
+      <c r="K195" s="3"/>
+      <c r="L195" s="3"/>
+      <c r="M195" s="3"/>
+      <c r="N195" s="3"/>
+      <c r="O195" s="3"/>
+      <c r="P195" s="11"/>
+    </row>
+    <row r="196" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="11"/>
+      <c r="B196" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C195" s="17" t="s">
+      <c r="C196" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="D195" s="17"/>
-      <c r="E195" s="17"/>
-      <c r="F195" s="17"/>
-      <c r="G195" s="17"/>
-      <c r="H195" s="17"/>
-      <c r="I195" s="17"/>
-      <c r="J195" s="17"/>
-      <c r="K195" s="17"/>
-      <c r="L195" s="17"/>
-      <c r="M195" s="17"/>
-      <c r="N195" s="17"/>
-      <c r="O195" s="17"/>
-      <c r="P195" s="17"/>
-    </row>
-    <row r="196" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A196" s="3"/>
-      <c r="B196" s="3"/>
-      <c r="C196" s="3"/>
-      <c r="D196" s="16"/>
-      <c r="E196" s="11"/>
-      <c r="F196" s="11"/>
-      <c r="G196" s="11"/>
-      <c r="H196" s="11"/>
-      <c r="I196" s="11"/>
-      <c r="J196" s="3"/>
-      <c r="K196" s="3"/>
-      <c r="L196" s="3"/>
-      <c r="M196" s="3"/>
-      <c r="N196" s="3"/>
-      <c r="O196" s="3"/>
-      <c r="P196" s="11"/>
+      <c r="D196" s="17"/>
+      <c r="E196" s="17"/>
+      <c r="F196" s="17"/>
+      <c r="G196" s="17"/>
+      <c r="H196" s="17"/>
+      <c r="I196" s="17"/>
+      <c r="J196" s="17"/>
+      <c r="K196" s="17"/>
+      <c r="L196" s="17"/>
+      <c r="M196" s="17"/>
+      <c r="N196" s="17"/>
+      <c r="O196" s="17"/>
+      <c r="P196" s="17"/>
     </row>
     <row r="197" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A197" s="3"/>
@@ -6093,19 +6106,19 @@
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
-      <c r="D198" s="3"/>
-      <c r="E198" s="3"/>
-      <c r="F198" s="17"/>
-      <c r="G198" s="3"/>
-      <c r="H198" s="3"/>
-      <c r="I198" s="3"/>
+      <c r="D198" s="16"/>
+      <c r="E198" s="11"/>
+      <c r="F198" s="11"/>
+      <c r="G198" s="11"/>
+      <c r="H198" s="11"/>
+      <c r="I198" s="11"/>
       <c r="J198" s="3"/>
       <c r="K198" s="3"/>
       <c r="L198" s="3"/>
       <c r="M198" s="3"/>
       <c r="N198" s="3"/>
       <c r="O198" s="3"/>
-      <c r="P198" s="3"/>
+      <c r="P198" s="11"/>
     </row>
     <row r="199" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A199" s="3"/>
@@ -6113,7 +6126,7 @@
       <c r="C199" s="3"/>
       <c r="D199" s="3"/>
       <c r="E199" s="3"/>
-      <c r="F199" s="11"/>
+      <c r="F199" s="17"/>
       <c r="G199" s="3"/>
       <c r="H199" s="3"/>
       <c r="I199" s="3"/>
@@ -6149,7 +6162,7 @@
       <c r="C201" s="3"/>
       <c r="D201" s="3"/>
       <c r="E201" s="3"/>
-      <c r="F201" s="17"/>
+      <c r="F201" s="11"/>
       <c r="G201" s="3"/>
       <c r="H201" s="3"/>
       <c r="I201" s="3"/>
@@ -6167,7 +6180,7 @@
       <c r="C202" s="3"/>
       <c r="D202" s="3"/>
       <c r="E202" s="3"/>
-      <c r="F202" s="11"/>
+      <c r="F202" s="17"/>
       <c r="G202" s="3"/>
       <c r="H202" s="3"/>
       <c r="I202" s="3"/>
@@ -6203,7 +6216,7 @@
       <c r="C204" s="3"/>
       <c r="D204" s="3"/>
       <c r="E204" s="3"/>
-      <c r="F204" s="3"/>
+      <c r="F204" s="11"/>
       <c r="G204" s="3"/>
       <c r="H204" s="3"/>
       <c r="I204" s="3"/>
@@ -6287,58 +6300,73 @@
       <c r="O208" s="3"/>
       <c r="P208" s="3"/>
     </row>
-    <row r="209" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A209" s="3"/>
+      <c r="B209" s="3"/>
       <c r="C209" s="3"/>
+      <c r="D209" s="3"/>
+      <c r="E209" s="3"/>
       <c r="F209" s="3"/>
-    </row>
-    <row r="210" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="G209" s="3"/>
+      <c r="H209" s="3"/>
+      <c r="I209" s="3"/>
+      <c r="J209" s="3"/>
+      <c r="K209" s="3"/>
+      <c r="L209" s="3"/>
+      <c r="M209" s="3"/>
+      <c r="N209" s="3"/>
+      <c r="O209" s="3"/>
+      <c r="P209" s="3"/>
+    </row>
+    <row r="210" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C210" s="3"/>
       <c r="F210" s="3"/>
     </row>
-    <row r="211" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C211" s="3"/>
       <c r="F211" s="3"/>
     </row>
-    <row r="212" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C212" s="3"/>
       <c r="F212" s="3"/>
     </row>
-    <row r="213" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C213" s="3"/>
       <c r="F213" s="3"/>
     </row>
-    <row r="214" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C214" s="3"/>
       <c r="F214" s="3"/>
     </row>
-    <row r="215" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C215" s="3"/>
-    </row>
-    <row r="216" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="F215" s="3"/>
+    </row>
+    <row r="216" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C216" s="3"/>
     </row>
-    <row r="217" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C217" s="3"/>
     </row>
-    <row r="218" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C218" s="3"/>
     </row>
-    <row r="219" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C219" s="3"/>
     </row>
-    <row r="220" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C220" s="3"/>
     </row>
-    <row r="221" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C221" s="3"/>
     </row>
-    <row r="222" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C222" s="3"/>
     </row>
-    <row r="223" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C223" s="3"/>
     </row>
-    <row r="224" spans="3:6" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C224" s="3"/>
     </row>
     <row r="225" spans="3:3" x14ac:dyDescent="0.25">
@@ -8813,28 +8841,31 @@
     <row r="1048" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C1048" s="3"/>
     </row>
+    <row r="1049" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C1049" s="3"/>
+    </row>
   </sheetData>
   <sheetProtection formatCells="0" formatRows="0" insertRows="0" insertHyperlinks="0" deleteRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="B10:P197" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="B10:P198" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="F1:P6"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="9">
-    <dataValidation allowBlank="1" showInputMessage="1" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C144 C189 C192 C195" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Object Code value" error="The Object code value shall be:_x000a_VARIABLE_x000a_RECORD_x000a_ARRAY" sqref="C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C36:C143 C145:C188 C190:C191 C193:C194 C196:C208" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation allowBlank="1" showInputMessage="1" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C144 C190 C193 C196" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Object Code value" error="The Object code value shall be:_x000a_VARIABLE_x000a_RECORD_x000a_ARRAY" sqref="C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C36:C143 C145:C189 C191:C192 C194:C195 C197:C209" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Category" error="The value for the entry category shall be _x000a_M : (mandatory)_x000a_O : (optional) _x000a_C : (conditional)" sqref="J36 J193:J194 J196:J208 J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J40:J143 J145:J188 J190:J191" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Category" error="The value for the entry category shall be _x000a_M : (mandatory)_x000a_O : (optional) _x000a_C : (conditional)" sqref="J36 J194:J195 J197:J209 J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J40:J143 J145:J189 J191:J192" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"M,O,C"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Backup/Setting Flag" error="The entry flag shall be_x000a_B : (Backup)_x000a_S : (Setting)" sqref="K36 K193:K194 K196:K208 K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K40:K143 K145:K188 K190:K191" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Backup/Setting Flag" error="The entry flag shall be_x000a_B : (Backup)_x000a_S : (Setting)" sqref="K36 K194:K195 K197:K209 K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K40:K143 K145:K189 K191:K192" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"B,S"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M36:O36 M193:O194 M12:O13 M18:O19 M24:O25 M30:O31 M40:O143 M190:O191 M196:O197 M15:O16 M21:O22 M27:O28 M33:O34 M145:O188" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M36:O36 M194:O195 M12:O13 M18:O19 M24:O25 M30:O31 M40:O143 M191:O192 M197:O198 M15:O16 M21:O22 M27:O28 M33:O34 M145:O189" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"rx,tx"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C209:C1048" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C210:C1049" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J37:J39" xr:uid="{20805EC6-BF85-484F-8728-8A67EE77DC8F}">

</xml_diff>

<commit_message>
1. update ethercat xml file 2. modify uart protocol thread priority 3. add debug interface to simulate dose plan data
</commit_message>
<xml_diff>
--- a/ArmCoreV1_QSPI/SSCProject/lan9252_app.xlsx
+++ b/ArmCoreV1_QSPI/SSCProject/lan9252_app.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\WORK\arm_core_develop\bgm_arm_io_develop\FW-ArmCore\ArmCoreV1_QSPI\SSCProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhong\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <workbookProtection lockStructure="1"/>
@@ -16,8 +16,8 @@
     <sheet name="Profile" sheetId="11" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Profile!$B$10:$P$76</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Profile!$B$1:$P$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Profile!$B$10:$P$93</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Profile!$B$1:$P$94</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="119">
   <si>
     <t>Device Profile:</t>
   </si>
@@ -385,6 +385,423 @@
   </si>
   <si>
     <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nU16_NotReadyEvent</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DINT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>In</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>U32_WaringInterlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nU32_MinorInterlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_SeriousInterlock</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>R</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EAL</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_PrimaryDoseTotalActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_SecondaryDoseTotalActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_PrimaryDoseRateActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nF_SecondaryDoseRateActual</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RM IO FSM State</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RM IO Interlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_DoseAInterlock</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>InU32_Dose</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Interlock</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DOSEA</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DOSEB</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>DOSEB</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>REAL</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_DoseAFsmState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_DoseBFsmState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>U</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DINT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>R</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EAL</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>OutU8_RequireState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utU8_BeamId</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>InU8_BeamI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>d</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utU16_RadiationIndex</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>R</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EAL</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>utF_GantryPosition</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>UDINT</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>UDINT</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>OutU32_InterlockOverride</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>OutU32_UnreadyOveride</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>REAL</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_BeamOnTime</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">ARM IO First Trigger Out start count </t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>UDINT</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_AfcState</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>UDINT</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_DoseAErrorCode</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_DoseBErrorCode</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
       <t>U</t>
     </r>
     <r>
@@ -402,7 +819,7 @@
   </si>
   <si>
     <r>
-      <t>I</t>
+      <t>U</t>
     </r>
     <r>
       <rPr>
@@ -413,13 +830,21 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>nU16_NotReadyEvent</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>U</t>
+      <t>SINT</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>USINT</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_AfcPositionCurrent</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>0</t>
     </r>
     <r>
       <rPr>
@@ -430,13 +855,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>DINT</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>In</t>
+      <t>: stop  1: run</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>0</t>
     </r>
     <r>
       <rPr>
@@ -447,9 +872,28 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>U32_WaringInterlock</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
+      <t>: no fault  1: fault</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_EpsFaultStop</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_EpsFaultCode</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_EpsCurrentOutput</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_EpsPowerOutput</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>REAL</t>
   </si>
   <si>
     <r>
@@ -464,17 +908,13 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>nU32_MinorInterlock</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>InU32_SeriousInterlock</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>R</t>
+      <t>nF_EpsVersion</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>InF_</t>
     </r>
     <r>
       <rPr>
@@ -485,13 +925,55 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>EAL</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>I</t>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>psVersion</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_EpsRunStatus</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_VpsRunStatus</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU8_VpsFaultStop</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InU32_VpsFaultCode</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_EpsVoltageOutput</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_VpsVoltageOutput</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_VpsCurrentOutput</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>InF_VpsPowerVoltage</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>In</t>
     </r>
     <r>
       <rPr>
@@ -502,311 +984,8 @@
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
-      <t>nF_PrimaryDoseTotalActual</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>I</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>nF_SecondaryDoseTotalActual</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>I</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>nF_PrimaryDoseRateActual</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>I</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>nF_SecondaryDoseRateActual</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RM IO FSM State</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RM IO Interlock</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>InU32_DoseAInterlock</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>InU32_Dose</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>B</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Interlock</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>DOSEA</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>DOSEB</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>DOSEB</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>REAL</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>InU8_DoseAFsmState</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>InU8_DoseBFsmState</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>U</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>DINT</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>R</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>EAL</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>InF_AfcPositionCurrent</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>OutU8_RequireState</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>O</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>utU8_BeamId</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>InU8_BeamI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>d</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>O</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>utU16_RadiationIndex</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>R</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>EAL</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>O</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>utF_GantryPosition</t>
-    </r>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>UDINT</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>UDINT</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>OutU32_InterlockOverride</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>OutU32_UnreadyOveride</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>REAL</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>InF_BeamOnTime</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">ARM IO First Trigger Out start count </t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>UDINT</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>InU32_AfcState</t>
+      <t>F_SF6Pressure</t>
+    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -1257,7 +1436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T927"/>
+  <dimension ref="A1:T944"/>
   <sheetFormatPr defaultColWidth="10.7265625" defaultRowHeight="14" outlineLevelRow="1"/>
   <cols>
     <col min="1" max="1" width="3.81640625" style="2" customWidth="1"/>
@@ -2062,7 +2241,7 @@
       <c r="N37" s="3"/>
       <c r="O37" s="3"/>
       <c r="P37" s="21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:16" customFormat="1">
@@ -2076,7 +2255,7 @@
         <v>42</v>
       </c>
       <c r="F38" s="21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G38" s="11"/>
       <c r="H38" s="11"/>
@@ -2121,10 +2300,10 @@
         <v>4</v>
       </c>
       <c r="E40" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="F40" s="21" t="s">
         <v>57</v>
-      </c>
-      <c r="F40" s="21" t="s">
-        <v>58</v>
       </c>
       <c r="G40" s="11"/>
       <c r="H40" s="11"/>
@@ -2145,10 +2324,10 @@
         <v>5</v>
       </c>
       <c r="E41" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="F41" s="21" t="s">
         <v>59</v>
-      </c>
-      <c r="F41" s="21" t="s">
-        <v>60</v>
       </c>
       <c r="G41" s="11"/>
       <c r="H41" s="11"/>
@@ -2169,10 +2348,10 @@
         <v>6</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F42" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G42" s="11"/>
       <c r="H42" s="11"/>
@@ -2193,10 +2372,10 @@
         <v>7</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F43" s="21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G43" s="11"/>
       <c r="H43" s="11"/>
@@ -2208,7 +2387,7 @@
       <c r="N43" s="3"/>
       <c r="O43" s="3"/>
       <c r="P43" s="21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44" spans="1:16" customFormat="1">
@@ -2219,10 +2398,10 @@
         <v>8</v>
       </c>
       <c r="E44" s="21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F44" s="21" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G44" s="11"/>
       <c r="H44" s="11"/>
@@ -2234,7 +2413,7 @@
       <c r="N44" s="3"/>
       <c r="O44" s="3"/>
       <c r="P44" s="21" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45" spans="1:16" customFormat="1">
@@ -2245,10 +2424,10 @@
         <v>9</v>
       </c>
       <c r="E45" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="F45" s="21" t="s">
         <v>63</v>
-      </c>
-      <c r="F45" s="21" t="s">
-        <v>64</v>
       </c>
       <c r="G45" s="11"/>
       <c r="H45" s="11"/>
@@ -2260,7 +2439,7 @@
       <c r="N45" s="3"/>
       <c r="O45" s="3"/>
       <c r="P45" s="21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="46" spans="1:16" customFormat="1">
@@ -2271,10 +2450,10 @@
         <v>10</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F46" s="21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G46" s="11"/>
       <c r="H46" s="11"/>
@@ -2286,7 +2465,7 @@
       <c r="N46" s="3"/>
       <c r="O46" s="3"/>
       <c r="P46" s="21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:16" customFormat="1">
@@ -2297,10 +2476,10 @@
         <v>11</v>
       </c>
       <c r="E47" s="21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F47" s="21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G47" s="11"/>
       <c r="H47" s="11"/>
@@ -2312,7 +2491,7 @@
       <c r="N47" s="3"/>
       <c r="O47" s="3"/>
       <c r="P47" s="21" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="48" spans="1:16" customFormat="1">
@@ -2323,10 +2502,10 @@
         <v>12</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F48" s="21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G48" s="11"/>
       <c r="H48" s="11"/>
@@ -2338,7 +2517,7 @@
       <c r="N48" s="3"/>
       <c r="O48" s="3"/>
       <c r="P48" s="21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" spans="1:16" customFormat="1">
@@ -2349,10 +2528,10 @@
         <v>13</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>55</v>
+        <v>98</v>
       </c>
       <c r="F49" s="21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G49" s="11"/>
       <c r="H49" s="11"/>
@@ -2376,7 +2555,7 @@
         <v>55</v>
       </c>
       <c r="F50" s="21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G50" s="11"/>
       <c r="H50" s="11"/>
@@ -2397,10 +2576,10 @@
         <v>15</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F51" s="21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G51" s="11"/>
       <c r="H51" s="11"/>
@@ -2421,10 +2600,10 @@
         <v>16</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F52" s="21" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G52" s="11"/>
       <c r="H52" s="11"/>
@@ -2469,10 +2648,10 @@
         <v>18</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F54" s="21" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="G54" s="11"/>
       <c r="H54" s="11"/>
@@ -2489,9 +2668,15 @@
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
-      <c r="D55" s="16"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="11"/>
+      <c r="D55" s="16">
+        <v>19</v>
+      </c>
+      <c r="E55" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="F55" s="21" t="s">
+        <v>93</v>
+      </c>
       <c r="G55" s="11"/>
       <c r="H55" s="11"/>
       <c r="I55" s="11"/>
@@ -2507,9 +2692,15 @@
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
-      <c r="D56" s="16"/>
-      <c r="E56" s="11"/>
-      <c r="F56" s="11"/>
+      <c r="D56" s="16">
+        <v>20</v>
+      </c>
+      <c r="E56" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F56" s="21" t="s">
+        <v>100</v>
+      </c>
       <c r="G56" s="11"/>
       <c r="H56" s="11"/>
       <c r="I56" s="11"/>
@@ -2521,40 +2712,42 @@
       <c r="O56" s="3"/>
       <c r="P56" s="11"/>
     </row>
-    <row r="57" spans="1:16" s="1" customFormat="1">
-      <c r="A57" s="11"/>
-      <c r="B57" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C57" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="D57" s="17"/>
-      <c r="E57" s="17"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="17"/>
-      <c r="O57" s="17"/>
-      <c r="P57" s="17"/>
-    </row>
-    <row r="58" spans="1:16">
+    <row r="57" spans="1:16" customFormat="1">
+      <c r="A57" s="3"/>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="16">
+        <v>21</v>
+      </c>
+      <c r="E57" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F57" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+      <c r="L57" s="3"/>
+      <c r="M57" s="3"/>
+      <c r="N57" s="3"/>
+      <c r="O57" s="3"/>
+      <c r="P57" s="11"/>
+    </row>
+    <row r="58" spans="1:16" customFormat="1">
       <c r="A58" s="3"/>
-      <c r="B58" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D58" s="16"/>
-      <c r="E58" s="11"/>
-      <c r="F58" s="11" t="s">
-        <v>47</v>
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="16">
+        <v>22</v>
+      </c>
+      <c r="E58" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="F58" s="21" t="s">
+        <v>110</v>
       </c>
       <c r="G58" s="11"/>
       <c r="H58" s="11"/>
@@ -2565,20 +2758,22 @@
       <c r="M58" s="3"/>
       <c r="N58" s="3"/>
       <c r="O58" s="3"/>
-      <c r="P58" s="11"/>
+      <c r="P58" s="21" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="59" spans="1:16" customFormat="1">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="16">
-        <v>1</v>
-      </c>
-      <c r="E59" s="11" t="s">
-        <v>42</v>
+        <v>23</v>
+      </c>
+      <c r="E59" s="21" t="s">
+        <v>99</v>
       </c>
       <c r="F59" s="21" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="G59" s="11"/>
       <c r="H59" s="11"/>
@@ -2589,20 +2784,22 @@
       <c r="M59" s="3"/>
       <c r="N59" s="3"/>
       <c r="O59" s="3"/>
-      <c r="P59" s="11"/>
+      <c r="P59" s="21" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="60" spans="1:16" customFormat="1">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="16">
-        <v>2</v>
-      </c>
-      <c r="E60" s="11" t="s">
-        <v>42</v>
+        <v>24</v>
+      </c>
+      <c r="E60" s="21" t="s">
+        <v>85</v>
       </c>
       <c r="F60" s="21" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="G60" s="11"/>
       <c r="H60" s="11"/>
@@ -2613,20 +2810,20 @@
       <c r="M60" s="3"/>
       <c r="N60" s="3"/>
       <c r="O60" s="3"/>
-      <c r="P60" s="11"/>
+      <c r="P60" s="21"/>
     </row>
     <row r="61" spans="1:16" customFormat="1">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
       <c r="D61" s="16">
-        <v>3</v>
-      </c>
-      <c r="E61" s="11" t="s">
-        <v>43</v>
+        <v>25</v>
+      </c>
+      <c r="E61" s="21" t="s">
+        <v>74</v>
       </c>
       <c r="F61" s="21" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="G61" s="11"/>
       <c r="H61" s="11"/>
@@ -2644,13 +2841,13 @@
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
       <c r="D62" s="16">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="E62" s="21" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="F62" s="21" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="G62" s="11"/>
       <c r="H62" s="11"/>
@@ -2668,13 +2865,13 @@
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
       <c r="D63" s="16">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="E63" s="21" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="F63" s="21" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="G63" s="11"/>
       <c r="H63" s="11"/>
@@ -2692,13 +2889,13 @@
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
       <c r="D64" s="16">
-        <v>6</v>
-      </c>
-      <c r="E64" s="21" t="s">
-        <v>85</v>
+        <v>28</v>
+      </c>
+      <c r="E64" s="11" t="s">
+        <v>107</v>
       </c>
       <c r="F64" s="21" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="G64" s="11"/>
       <c r="H64" s="11"/>
@@ -2715,9 +2912,15 @@
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
-      <c r="D65" s="16"/>
-      <c r="E65" s="11"/>
-      <c r="F65" s="11"/>
+      <c r="D65" s="16">
+        <v>29</v>
+      </c>
+      <c r="E65" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="F65" s="21" t="s">
+        <v>111</v>
+      </c>
       <c r="G65" s="11"/>
       <c r="H65" s="11"/>
       <c r="I65" s="11"/>
@@ -2733,9 +2936,15 @@
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
-      <c r="D66" s="16"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="11"/>
+      <c r="D66" s="16">
+        <v>30</v>
+      </c>
+      <c r="E66" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="F66" s="21" t="s">
+        <v>112</v>
+      </c>
       <c r="G66" s="11"/>
       <c r="H66" s="11"/>
       <c r="I66" s="11"/>
@@ -2751,9 +2960,15 @@
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
-      <c r="D67" s="16"/>
-      <c r="E67" s="11"/>
-      <c r="F67" s="11"/>
+      <c r="D67" s="16">
+        <v>31</v>
+      </c>
+      <c r="E67" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="F67" s="21" t="s">
+        <v>113</v>
+      </c>
       <c r="G67" s="11"/>
       <c r="H67" s="11"/>
       <c r="I67" s="11"/>
@@ -2765,35 +2980,43 @@
       <c r="O67" s="3"/>
       <c r="P67" s="11"/>
     </row>
-    <row r="68" spans="1:16" s="1" customFormat="1">
-      <c r="A68" s="11"/>
-      <c r="B68" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="C68" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="D68" s="17"/>
-      <c r="E68" s="17"/>
-      <c r="F68" s="18"/>
-      <c r="G68" s="17"/>
-      <c r="H68" s="17"/>
-      <c r="I68" s="17"/>
-      <c r="J68" s="17"/>
-      <c r="K68" s="17"/>
-      <c r="L68" s="17"/>
-      <c r="M68" s="17"/>
-      <c r="N68" s="17"/>
-      <c r="O68" s="17"/>
-      <c r="P68" s="17"/>
-    </row>
-    <row r="69" spans="1:16">
+    <row r="68" spans="1:16" customFormat="1">
+      <c r="A68" s="3"/>
+      <c r="B68" s="3"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="16">
+        <v>32</v>
+      </c>
+      <c r="E68" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F68" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+      <c r="J68" s="3"/>
+      <c r="K68" s="3"/>
+      <c r="L68" s="3"/>
+      <c r="M68" s="3"/>
+      <c r="N68" s="3"/>
+      <c r="O68" s="3"/>
+      <c r="P68" s="11"/>
+    </row>
+    <row r="69" spans="1:16" customFormat="1">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
-      <c r="D69" s="16"/>
-      <c r="E69" s="11"/>
-      <c r="F69" s="11"/>
+      <c r="D69" s="16">
+        <v>33</v>
+      </c>
+      <c r="E69" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F69" s="21" t="s">
+        <v>116</v>
+      </c>
       <c r="G69" s="11"/>
       <c r="H69" s="11"/>
       <c r="I69" s="11"/>
@@ -2805,13 +3028,19 @@
       <c r="O69" s="3"/>
       <c r="P69" s="11"/>
     </row>
-    <row r="70" spans="1:16">
+    <row r="70" spans="1:16" customFormat="1">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
-      <c r="D70" s="16"/>
-      <c r="E70" s="11"/>
-      <c r="F70" s="11"/>
+      <c r="D70" s="16">
+        <v>34</v>
+      </c>
+      <c r="E70" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F70" s="21" t="s">
+        <v>117</v>
+      </c>
       <c r="G70" s="11"/>
       <c r="H70" s="11"/>
       <c r="I70" s="11"/>
@@ -2823,34 +3052,36 @@
       <c r="O70" s="3"/>
       <c r="P70" s="11"/>
     </row>
-    <row r="71" spans="1:16" s="1" customFormat="1">
-      <c r="A71" s="11"/>
-      <c r="B71" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C71" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="D71" s="17"/>
-      <c r="E71" s="17"/>
-      <c r="F71" s="11"/>
-      <c r="G71" s="17"/>
-      <c r="H71" s="17"/>
-      <c r="I71" s="17"/>
-      <c r="J71" s="17"/>
-      <c r="K71" s="17"/>
-      <c r="L71" s="17"/>
-      <c r="M71" s="17"/>
-      <c r="N71" s="17"/>
-      <c r="O71" s="17"/>
-      <c r="P71" s="17"/>
-    </row>
-    <row r="72" spans="1:16">
+    <row r="71" spans="1:16" customFormat="1">
+      <c r="A71" s="3"/>
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="16">
+        <v>35</v>
+      </c>
+      <c r="E71" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F71" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="G71" s="11"/>
+      <c r="H71" s="11"/>
+      <c r="I71" s="11"/>
+      <c r="J71" s="3"/>
+      <c r="K71" s="3"/>
+      <c r="L71" s="3"/>
+      <c r="M71" s="3"/>
+      <c r="N71" s="3"/>
+      <c r="O71" s="3"/>
+      <c r="P71" s="11"/>
+    </row>
+    <row r="72" spans="1:16" customFormat="1">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
       <c r="D72" s="16"/>
-      <c r="E72" s="11"/>
+      <c r="E72" s="21"/>
       <c r="F72" s="11"/>
       <c r="G72" s="11"/>
       <c r="H72" s="11"/>
@@ -2863,7 +3094,7 @@
       <c r="O72" s="3"/>
       <c r="P72" s="11"/>
     </row>
-    <row r="73" spans="1:16">
+    <row r="73" spans="1:16" customFormat="1">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -2884,10 +3115,10 @@
     <row r="74" spans="1:16" s="1" customFormat="1">
       <c r="A74" s="11"/>
       <c r="B74" s="17" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C74" s="17" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D74" s="17"/>
       <c r="E74" s="17"/>
@@ -2905,11 +3136,17 @@
     </row>
     <row r="75" spans="1:16">
       <c r="A75" s="3"/>
-      <c r="B75" s="3"/>
-      <c r="C75" s="3"/>
+      <c r="B75" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="D75" s="16"/>
       <c r="E75" s="11"/>
-      <c r="F75" s="11"/>
+      <c r="F75" s="11" t="s">
+        <v>47</v>
+      </c>
       <c r="G75" s="11"/>
       <c r="H75" s="11"/>
       <c r="I75" s="11"/>
@@ -2921,13 +3158,19 @@
       <c r="O75" s="3"/>
       <c r="P75" s="11"/>
     </row>
-    <row r="76" spans="1:16">
+    <row r="76" spans="1:16" customFormat="1">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
-      <c r="D76" s="16"/>
-      <c r="E76" s="11"/>
-      <c r="F76" s="11"/>
+      <c r="D76" s="16">
+        <v>1</v>
+      </c>
+      <c r="E76" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F76" s="21" t="s">
+        <v>79</v>
+      </c>
       <c r="G76" s="11"/>
       <c r="H76" s="11"/>
       <c r="I76" s="11"/>
@@ -2939,283 +3182,580 @@
       <c r="O76" s="3"/>
       <c r="P76" s="11"/>
     </row>
-    <row r="77" spans="1:16">
+    <row r="77" spans="1:16" customFormat="1">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
-      <c r="D77" s="3"/>
-      <c r="E77" s="3"/>
-      <c r="F77" s="17"/>
-      <c r="G77" s="3"/>
-      <c r="H77" s="3"/>
-      <c r="I77" s="3"/>
+      <c r="D77" s="16">
+        <v>2</v>
+      </c>
+      <c r="E77" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="F77" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="G77" s="11"/>
+      <c r="H77" s="11"/>
+      <c r="I77" s="11"/>
       <c r="J77" s="3"/>
       <c r="K77" s="3"/>
       <c r="L77" s="3"/>
       <c r="M77" s="3"/>
       <c r="N77" s="3"/>
       <c r="O77" s="3"/>
-      <c r="P77" s="3"/>
-    </row>
-    <row r="78" spans="1:16">
+      <c r="P77" s="11"/>
+    </row>
+    <row r="78" spans="1:16" customFormat="1">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
-      <c r="D78" s="3"/>
-      <c r="E78" s="3"/>
-      <c r="F78" s="11"/>
-      <c r="G78" s="3"/>
-      <c r="H78" s="3"/>
-      <c r="I78" s="3"/>
+      <c r="D78" s="16">
+        <v>3</v>
+      </c>
+      <c r="E78" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F78" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="G78" s="11"/>
+      <c r="H78" s="11"/>
+      <c r="I78" s="11"/>
       <c r="J78" s="3"/>
       <c r="K78" s="3"/>
       <c r="L78" s="3"/>
       <c r="M78" s="3"/>
       <c r="N78" s="3"/>
       <c r="O78" s="3"/>
-      <c r="P78" s="3"/>
-    </row>
-    <row r="79" spans="1:16">
+      <c r="P78" s="11"/>
+    </row>
+    <row r="79" spans="1:16" customFormat="1">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
-      <c r="D79" s="3"/>
-      <c r="E79" s="3"/>
-      <c r="F79" s="11"/>
-      <c r="G79" s="3"/>
-      <c r="H79" s="3"/>
-      <c r="I79" s="3"/>
+      <c r="D79" s="16">
+        <v>4</v>
+      </c>
+      <c r="E79" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="F79" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G79" s="11"/>
+      <c r="H79" s="11"/>
+      <c r="I79" s="11"/>
       <c r="J79" s="3"/>
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
       <c r="M79" s="3"/>
       <c r="N79" s="3"/>
       <c r="O79" s="3"/>
-      <c r="P79" s="3"/>
-    </row>
-    <row r="80" spans="1:16">
+      <c r="P79" s="11"/>
+    </row>
+    <row r="80" spans="1:16" customFormat="1">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
-      <c r="D80" s="3"/>
-      <c r="E80" s="3"/>
-      <c r="F80" s="17"/>
-      <c r="G80" s="3"/>
-      <c r="H80" s="3"/>
-      <c r="I80" s="3"/>
+      <c r="D80" s="16">
+        <v>5</v>
+      </c>
+      <c r="E80" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="F80" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="G80" s="11"/>
+      <c r="H80" s="11"/>
+      <c r="I80" s="11"/>
       <c r="J80" s="3"/>
       <c r="K80" s="3"/>
       <c r="L80" s="3"/>
       <c r="M80" s="3"/>
       <c r="N80" s="3"/>
       <c r="O80" s="3"/>
-      <c r="P80" s="3"/>
-    </row>
-    <row r="81" spans="1:16">
+      <c r="P80" s="11"/>
+    </row>
+    <row r="81" spans="1:16" customFormat="1">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
-      <c r="D81" s="3"/>
-      <c r="E81" s="3"/>
-      <c r="F81" s="11"/>
-      <c r="G81" s="3"/>
-      <c r="H81" s="3"/>
-      <c r="I81" s="3"/>
+      <c r="D81" s="16">
+        <v>6</v>
+      </c>
+      <c r="E81" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="F81" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="G81" s="11"/>
+      <c r="H81" s="11"/>
+      <c r="I81" s="11"/>
       <c r="J81" s="3"/>
       <c r="K81" s="3"/>
       <c r="L81" s="3"/>
       <c r="M81" s="3"/>
       <c r="N81" s="3"/>
       <c r="O81" s="3"/>
-      <c r="P81" s="3"/>
-    </row>
-    <row r="82" spans="1:16">
+      <c r="P81" s="11"/>
+    </row>
+    <row r="82" spans="1:16" customFormat="1">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
-      <c r="D82" s="3"/>
-      <c r="E82" s="3"/>
+      <c r="D82" s="16"/>
+      <c r="E82" s="11"/>
       <c r="F82" s="11"/>
-      <c r="G82" s="3"/>
-      <c r="H82" s="3"/>
-      <c r="I82" s="3"/>
+      <c r="G82" s="11"/>
+      <c r="H82" s="11"/>
+      <c r="I82" s="11"/>
       <c r="J82" s="3"/>
       <c r="K82" s="3"/>
       <c r="L82" s="3"/>
       <c r="M82" s="3"/>
       <c r="N82" s="3"/>
       <c r="O82" s="3"/>
-      <c r="P82" s="3"/>
-    </row>
-    <row r="83" spans="1:16">
+      <c r="P82" s="11"/>
+    </row>
+    <row r="83" spans="1:16" customFormat="1">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
-      <c r="D83" s="3"/>
-      <c r="E83" s="3"/>
-      <c r="F83" s="3"/>
-      <c r="G83" s="3"/>
-      <c r="H83" s="3"/>
-      <c r="I83" s="3"/>
+      <c r="D83" s="16"/>
+      <c r="E83" s="11"/>
+      <c r="F83" s="11"/>
+      <c r="G83" s="11"/>
+      <c r="H83" s="11"/>
+      <c r="I83" s="11"/>
       <c r="J83" s="3"/>
       <c r="K83" s="3"/>
       <c r="L83" s="3"/>
       <c r="M83" s="3"/>
       <c r="N83" s="3"/>
       <c r="O83" s="3"/>
-      <c r="P83" s="3"/>
-    </row>
-    <row r="84" spans="1:16">
+      <c r="P83" s="11"/>
+    </row>
+    <row r="84" spans="1:16" customFormat="1">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
-      <c r="D84" s="3"/>
-      <c r="E84" s="3"/>
-      <c r="F84" s="3"/>
-      <c r="G84" s="3"/>
-      <c r="H84" s="3"/>
-      <c r="I84" s="3"/>
+      <c r="D84" s="16"/>
+      <c r="E84" s="11"/>
+      <c r="F84" s="11"/>
+      <c r="G84" s="11"/>
+      <c r="H84" s="11"/>
+      <c r="I84" s="11"/>
       <c r="J84" s="3"/>
       <c r="K84" s="3"/>
       <c r="L84" s="3"/>
       <c r="M84" s="3"/>
       <c r="N84" s="3"/>
       <c r="O84" s="3"/>
-      <c r="P84" s="3"/>
-    </row>
-    <row r="85" spans="1:16">
-      <c r="A85" s="3"/>
-      <c r="B85" s="3"/>
-      <c r="C85" s="3"/>
-      <c r="D85" s="3"/>
-      <c r="E85" s="3"/>
-      <c r="F85" s="3"/>
-      <c r="G85" s="3"/>
-      <c r="H85" s="3"/>
-      <c r="I85" s="3"/>
-      <c r="J85" s="3"/>
-      <c r="K85" s="3"/>
-      <c r="L85" s="3"/>
-      <c r="M85" s="3"/>
-      <c r="N85" s="3"/>
-      <c r="O85" s="3"/>
-      <c r="P85" s="3"/>
+      <c r="P84" s="11"/>
+    </row>
+    <row r="85" spans="1:16" s="1" customFormat="1">
+      <c r="A85" s="11"/>
+      <c r="B85" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C85" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D85" s="17"/>
+      <c r="E85" s="17"/>
+      <c r="F85" s="18"/>
+      <c r="G85" s="17"/>
+      <c r="H85" s="17"/>
+      <c r="I85" s="17"/>
+      <c r="J85" s="17"/>
+      <c r="K85" s="17"/>
+      <c r="L85" s="17"/>
+      <c r="M85" s="17"/>
+      <c r="N85" s="17"/>
+      <c r="O85" s="17"/>
+      <c r="P85" s="17"/>
     </row>
     <row r="86" spans="1:16">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
+      <c r="D86" s="16"/>
+      <c r="E86" s="11"/>
+      <c r="F86" s="11"/>
+      <c r="G86" s="11"/>
+      <c r="H86" s="11"/>
+      <c r="I86" s="11"/>
       <c r="J86" s="3"/>
       <c r="K86" s="3"/>
       <c r="L86" s="3"/>
       <c r="M86" s="3"/>
       <c r="N86" s="3"/>
       <c r="O86" s="3"/>
-      <c r="P86" s="3"/>
+      <c r="P86" s="11"/>
     </row>
     <row r="87" spans="1:16">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
-      <c r="D87" s="3"/>
-      <c r="E87" s="3"/>
-      <c r="F87" s="3"/>
-      <c r="G87" s="3"/>
-      <c r="H87" s="3"/>
-      <c r="I87" s="3"/>
+      <c r="D87" s="16"/>
+      <c r="E87" s="11"/>
+      <c r="F87" s="11"/>
+      <c r="G87" s="11"/>
+      <c r="H87" s="11"/>
+      <c r="I87" s="11"/>
       <c r="J87" s="3"/>
       <c r="K87" s="3"/>
       <c r="L87" s="3"/>
       <c r="M87" s="3"/>
       <c r="N87" s="3"/>
       <c r="O87" s="3"/>
-      <c r="P87" s="3"/>
-    </row>
-    <row r="88" spans="1:16">
-      <c r="C88" s="3"/>
-      <c r="F88" s="3"/>
+      <c r="P87" s="11"/>
+    </row>
+    <row r="88" spans="1:16" s="1" customFormat="1">
+      <c r="A88" s="11"/>
+      <c r="B88" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C88" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D88" s="17"/>
+      <c r="E88" s="17"/>
+      <c r="F88" s="11"/>
+      <c r="G88" s="17"/>
+      <c r="H88" s="17"/>
+      <c r="I88" s="17"/>
+      <c r="J88" s="17"/>
+      <c r="K88" s="17"/>
+      <c r="L88" s="17"/>
+      <c r="M88" s="17"/>
+      <c r="N88" s="17"/>
+      <c r="O88" s="17"/>
+      <c r="P88" s="17"/>
     </row>
     <row r="89" spans="1:16">
+      <c r="A89" s="3"/>
+      <c r="B89" s="3"/>
       <c r="C89" s="3"/>
-      <c r="F89" s="3"/>
+      <c r="D89" s="16"/>
+      <c r="E89" s="11"/>
+      <c r="F89" s="11"/>
+      <c r="G89" s="11"/>
+      <c r="H89" s="11"/>
+      <c r="I89" s="11"/>
+      <c r="J89" s="3"/>
+      <c r="K89" s="3"/>
+      <c r="L89" s="3"/>
+      <c r="M89" s="3"/>
+      <c r="N89" s="3"/>
+      <c r="O89" s="3"/>
+      <c r="P89" s="11"/>
     </row>
     <row r="90" spans="1:16">
+      <c r="A90" s="3"/>
+      <c r="B90" s="3"/>
       <c r="C90" s="3"/>
-      <c r="F90" s="3"/>
-    </row>
-    <row r="91" spans="1:16">
-      <c r="C91" s="3"/>
-      <c r="F91" s="3"/>
+      <c r="D90" s="16"/>
+      <c r="E90" s="11"/>
+      <c r="F90" s="11"/>
+      <c r="G90" s="11"/>
+      <c r="H90" s="11"/>
+      <c r="I90" s="11"/>
+      <c r="J90" s="3"/>
+      <c r="K90" s="3"/>
+      <c r="L90" s="3"/>
+      <c r="M90" s="3"/>
+      <c r="N90" s="3"/>
+      <c r="O90" s="3"/>
+      <c r="P90" s="11"/>
+    </row>
+    <row r="91" spans="1:16" s="1" customFormat="1">
+      <c r="A91" s="11"/>
+      <c r="B91" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C91" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D91" s="17"/>
+      <c r="E91" s="17"/>
+      <c r="F91" s="17"/>
+      <c r="G91" s="17"/>
+      <c r="H91" s="17"/>
+      <c r="I91" s="17"/>
+      <c r="J91" s="17"/>
+      <c r="K91" s="17"/>
+      <c r="L91" s="17"/>
+      <c r="M91" s="17"/>
+      <c r="N91" s="17"/>
+      <c r="O91" s="17"/>
+      <c r="P91" s="17"/>
     </row>
     <row r="92" spans="1:16">
+      <c r="A92" s="3"/>
+      <c r="B92" s="3"/>
       <c r="C92" s="3"/>
-      <c r="F92" s="3"/>
+      <c r="D92" s="16"/>
+      <c r="E92" s="11"/>
+      <c r="F92" s="11"/>
+      <c r="G92" s="11"/>
+      <c r="H92" s="11"/>
+      <c r="I92" s="11"/>
+      <c r="J92" s="3"/>
+      <c r="K92" s="3"/>
+      <c r="L92" s="3"/>
+      <c r="M92" s="3"/>
+      <c r="N92" s="3"/>
+      <c r="O92" s="3"/>
+      <c r="P92" s="11"/>
     </row>
     <row r="93" spans="1:16">
+      <c r="A93" s="3"/>
+      <c r="B93" s="3"/>
       <c r="C93" s="3"/>
-      <c r="F93" s="3"/>
+      <c r="D93" s="16"/>
+      <c r="E93" s="11"/>
+      <c r="F93" s="11"/>
+      <c r="G93" s="11"/>
+      <c r="H93" s="11"/>
+      <c r="I93" s="11"/>
+      <c r="J93" s="3"/>
+      <c r="K93" s="3"/>
+      <c r="L93" s="3"/>
+      <c r="M93" s="3"/>
+      <c r="N93" s="3"/>
+      <c r="O93" s="3"/>
+      <c r="P93" s="11"/>
     </row>
     <row r="94" spans="1:16">
+      <c r="A94" s="3"/>
+      <c r="B94" s="3"/>
       <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="17"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
+      <c r="I94" s="3"/>
+      <c r="J94" s="3"/>
+      <c r="K94" s="3"/>
+      <c r="L94" s="3"/>
+      <c r="M94" s="3"/>
+      <c r="N94" s="3"/>
+      <c r="O94" s="3"/>
+      <c r="P94" s="3"/>
     </row>
     <row r="95" spans="1:16">
+      <c r="A95" s="3"/>
+      <c r="B95" s="3"/>
       <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="11"/>
+      <c r="G95" s="3"/>
+      <c r="H95" s="3"/>
+      <c r="I95" s="3"/>
+      <c r="J95" s="3"/>
+      <c r="K95" s="3"/>
+      <c r="L95" s="3"/>
+      <c r="M95" s="3"/>
+      <c r="N95" s="3"/>
+      <c r="O95" s="3"/>
+      <c r="P95" s="3"/>
     </row>
     <row r="96" spans="1:16">
+      <c r="A96" s="3"/>
+      <c r="B96" s="3"/>
       <c r="C96" s="3"/>
-    </row>
-    <row r="97" spans="3:3">
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="11"/>
+      <c r="G96" s="3"/>
+      <c r="H96" s="3"/>
+      <c r="I96" s="3"/>
+      <c r="J96" s="3"/>
+      <c r="K96" s="3"/>
+      <c r="L96" s="3"/>
+      <c r="M96" s="3"/>
+      <c r="N96" s="3"/>
+      <c r="O96" s="3"/>
+      <c r="P96" s="3"/>
+    </row>
+    <row r="97" spans="1:16">
+      <c r="A97" s="3"/>
+      <c r="B97" s="3"/>
       <c r="C97" s="3"/>
-    </row>
-    <row r="98" spans="3:3">
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="17"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="3"/>
+      <c r="I97" s="3"/>
+      <c r="J97" s="3"/>
+      <c r="K97" s="3"/>
+      <c r="L97" s="3"/>
+      <c r="M97" s="3"/>
+      <c r="N97" s="3"/>
+      <c r="O97" s="3"/>
+      <c r="P97" s="3"/>
+    </row>
+    <row r="98" spans="1:16">
+      <c r="A98" s="3"/>
+      <c r="B98" s="3"/>
       <c r="C98" s="3"/>
-    </row>
-    <row r="99" spans="3:3">
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="11"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+      <c r="I98" s="3"/>
+      <c r="J98" s="3"/>
+      <c r="K98" s="3"/>
+      <c r="L98" s="3"/>
+      <c r="M98" s="3"/>
+      <c r="N98" s="3"/>
+      <c r="O98" s="3"/>
+      <c r="P98" s="3"/>
+    </row>
+    <row r="99" spans="1:16">
+      <c r="A99" s="3"/>
+      <c r="B99" s="3"/>
       <c r="C99" s="3"/>
-    </row>
-    <row r="100" spans="3:3">
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="11"/>
+      <c r="G99" s="3"/>
+      <c r="H99" s="3"/>
+      <c r="I99" s="3"/>
+      <c r="J99" s="3"/>
+      <c r="K99" s="3"/>
+      <c r="L99" s="3"/>
+      <c r="M99" s="3"/>
+      <c r="N99" s="3"/>
+      <c r="O99" s="3"/>
+      <c r="P99" s="3"/>
+    </row>
+    <row r="100" spans="1:16">
+      <c r="A100" s="3"/>
+      <c r="B100" s="3"/>
       <c r="C100" s="3"/>
-    </row>
-    <row r="101" spans="3:3">
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="3"/>
+      <c r="H100" s="3"/>
+      <c r="I100" s="3"/>
+      <c r="J100" s="3"/>
+      <c r="K100" s="3"/>
+      <c r="L100" s="3"/>
+      <c r="M100" s="3"/>
+      <c r="N100" s="3"/>
+      <c r="O100" s="3"/>
+      <c r="P100" s="3"/>
+    </row>
+    <row r="101" spans="1:16">
+      <c r="A101" s="3"/>
+      <c r="B101" s="3"/>
       <c r="C101" s="3"/>
-    </row>
-    <row r="102" spans="3:3">
+      <c r="D101" s="3"/>
+      <c r="E101" s="3"/>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+      <c r="I101" s="3"/>
+      <c r="J101" s="3"/>
+      <c r="K101" s="3"/>
+      <c r="L101" s="3"/>
+      <c r="M101" s="3"/>
+      <c r="N101" s="3"/>
+      <c r="O101" s="3"/>
+      <c r="P101" s="3"/>
+    </row>
+    <row r="102" spans="1:16">
+      <c r="A102" s="3"/>
+      <c r="B102" s="3"/>
       <c r="C102" s="3"/>
-    </row>
-    <row r="103" spans="3:3">
+      <c r="D102" s="3"/>
+      <c r="E102" s="3"/>
+      <c r="F102" s="3"/>
+      <c r="G102" s="3"/>
+      <c r="H102" s="3"/>
+      <c r="I102" s="3"/>
+      <c r="J102" s="3"/>
+      <c r="K102" s="3"/>
+      <c r="L102" s="3"/>
+      <c r="M102" s="3"/>
+      <c r="N102" s="3"/>
+      <c r="O102" s="3"/>
+      <c r="P102" s="3"/>
+    </row>
+    <row r="103" spans="1:16">
+      <c r="A103" s="3"/>
+      <c r="B103" s="3"/>
       <c r="C103" s="3"/>
-    </row>
-    <row r="104" spans="3:3">
+      <c r="D103" s="3"/>
+      <c r="E103" s="3"/>
+      <c r="F103" s="3"/>
+      <c r="G103" s="3"/>
+      <c r="H103" s="3"/>
+      <c r="I103" s="3"/>
+      <c r="J103" s="3"/>
+      <c r="K103" s="3"/>
+      <c r="L103" s="3"/>
+      <c r="M103" s="3"/>
+      <c r="N103" s="3"/>
+      <c r="O103" s="3"/>
+      <c r="P103" s="3"/>
+    </row>
+    <row r="104" spans="1:16">
+      <c r="A104" s="3"/>
+      <c r="B104" s="3"/>
       <c r="C104" s="3"/>
-    </row>
-    <row r="105" spans="3:3">
+      <c r="D104" s="3"/>
+      <c r="E104" s="3"/>
+      <c r="F104" s="3"/>
+      <c r="G104" s="3"/>
+      <c r="H104" s="3"/>
+      <c r="I104" s="3"/>
+      <c r="J104" s="3"/>
+      <c r="K104" s="3"/>
+      <c r="L104" s="3"/>
+      <c r="M104" s="3"/>
+      <c r="N104" s="3"/>
+      <c r="O104" s="3"/>
+      <c r="P104" s="3"/>
+    </row>
+    <row r="105" spans="1:16">
       <c r="C105" s="3"/>
-    </row>
-    <row r="106" spans="3:3">
+      <c r="F105" s="3"/>
+    </row>
+    <row r="106" spans="1:16">
       <c r="C106" s="3"/>
-    </row>
-    <row r="107" spans="3:3">
+      <c r="F106" s="3"/>
+    </row>
+    <row r="107" spans="1:16">
       <c r="C107" s="3"/>
-    </row>
-    <row r="108" spans="3:3">
+      <c r="F107" s="3"/>
+    </row>
+    <row r="108" spans="1:16">
       <c r="C108" s="3"/>
-    </row>
-    <row r="109" spans="3:3">
+      <c r="F108" s="3"/>
+    </row>
+    <row r="109" spans="1:16">
       <c r="C109" s="3"/>
-    </row>
-    <row r="110" spans="3:3">
+      <c r="F109" s="3"/>
+    </row>
+    <row r="110" spans="1:16">
       <c r="C110" s="3"/>
-    </row>
-    <row r="111" spans="3:3">
+      <c r="F110" s="3"/>
+    </row>
+    <row r="111" spans="1:16">
       <c r="C111" s="3"/>
     </row>
-    <row r="112" spans="3:3">
+    <row r="112" spans="1:16">
       <c r="C112" s="3"/>
     </row>
     <row r="113" spans="3:3">
@@ -5663,28 +6203,79 @@
     <row r="927" spans="3:3">
       <c r="C927" s="3"/>
     </row>
+    <row r="928" spans="3:3">
+      <c r="C928" s="3"/>
+    </row>
+    <row r="929" spans="3:3">
+      <c r="C929" s="3"/>
+    </row>
+    <row r="930" spans="3:3">
+      <c r="C930" s="3"/>
+    </row>
+    <row r="931" spans="3:3">
+      <c r="C931" s="3"/>
+    </row>
+    <row r="932" spans="3:3">
+      <c r="C932" s="3"/>
+    </row>
+    <row r="933" spans="3:3">
+      <c r="C933" s="3"/>
+    </row>
+    <row r="934" spans="3:3">
+      <c r="C934" s="3"/>
+    </row>
+    <row r="935" spans="3:3">
+      <c r="C935" s="3"/>
+    </row>
+    <row r="936" spans="3:3">
+      <c r="C936" s="3"/>
+    </row>
+    <row r="937" spans="3:3">
+      <c r="C937" s="3"/>
+    </row>
+    <row r="938" spans="3:3">
+      <c r="C938" s="3"/>
+    </row>
+    <row r="939" spans="3:3">
+      <c r="C939" s="3"/>
+    </row>
+    <row r="940" spans="3:3">
+      <c r="C940" s="3"/>
+    </row>
+    <row r="941" spans="3:3">
+      <c r="C941" s="3"/>
+    </row>
+    <row r="942" spans="3:3">
+      <c r="C942" s="3"/>
+    </row>
+    <row r="943" spans="3:3">
+      <c r="C943" s="3"/>
+    </row>
+    <row r="944" spans="3:3">
+      <c r="C944" s="3"/>
+    </row>
   </sheetData>
   <sheetProtection formatCells="0" formatRows="0" insertRows="0" insertHyperlinks="0" deleteRows="0" sort="0" autoFilter="0"/>
-  <autoFilter ref="B10:P76"/>
+  <autoFilter ref="B10:P93"/>
   <mergeCells count="1">
     <mergeCell ref="F1:P6"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation allowBlank="1" showInputMessage="1" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C57 C68 C71 C74"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Object Code value" error="The Object code value shall be:_x000a_VARIABLE_x000a_RECORD_x000a_ARRAY" sqref="C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C58:C67 C69:C70 C72:C73 C75:C87 C36:C56">
+    <dataValidation allowBlank="1" showInputMessage="1" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C74 C85 C88 C91"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Object Code value" error="The Object code value shall be:_x000a_VARIABLE_x000a_RECORD_x000a_ARRAY" sqref="C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C75:C84 C86:C87 C89:C90 C92:C104 C36:C73">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Category" error="The value for the entry category shall be _x000a_M : (mandatory)_x000a_O : (optional) _x000a_C : (conditional)" sqref="J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J58:J67 J69:J70 J72:J73 J75:J87 J36:J56">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Category" error="The value for the entry category shall be _x000a_M : (mandatory)_x000a_O : (optional) _x000a_C : (conditional)" sqref="J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J75:J84 J86:J87 J89:J90 J92:J104 J36:J73">
       <formula1>"M,O,C"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Backup/Setting Flag" error="The entry flag shall be_x000a_B : (Backup)_x000a_S : (Setting)" sqref="K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K58:K67 K69:K70 K72:K73 K75:K87 K36:K56">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Backup/Setting Flag" error="The entry flag shall be_x000a_B : (Backup)_x000a_S : (Setting)" sqref="K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K75:K84 K86:K87 K89:K90 K92:K104 K36:K73">
       <formula1>"B,S"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M12:O13 M18:O19 M24:O25 M30:O31 M69:O70 M75:O76 M15:O16 M21:O22 M27:O28 M33:O34 M72:O73 M58:O67 M36:O56">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M12:O13 M18:O19 M24:O25 M30:O31 M86:O87 M92:O93 M15:O16 M21:O22 M27:O28 M33:O34 M89:O90 M75:O84 M36:O73">
       <formula1>"rx,tx"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C88:C927">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C105:C944">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>